<commit_message>
library: publish NEH v9, Interior Plateau v6 and Southeastern Plains v1 under methodology 0.14
Northeastern Highlands v9 carries 23 curves of v8, rebuilds chlorophyll a
and large wood volume on the region's own stations, and adds total benthic
richness to Population support (31 metrics, 20 of 20 functions). Interior
Plateau v6 carries 22 curves of v5, rebuilds native fish richness and large
wood volume on the NARS-9 Southern Appalachians pool, and withholds
chlorophyll a (29 metrics, 20 of 20). Southeastern Plains v1 is the first
region the workflow built on its own (25 metrics, 19 of 20, Surface water
storage a documented gap confirmed at promote). All three are preliminary.
DEEP's registry, bundles and calculators are re-baked.
</commit_message>
<xml_diff>
--- a/apps/deep/www/calculators/interior-plateau.xlsx
+++ b/apps/deep/www/calculators/interior-plateau.xlsx
@@ -16,23 +16,23 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChartData" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="curve_key">'Reference'!$A$5:$A$34</definedName>
-    <definedName name="curve_x1">'Reference'!$G$5:$G$34</definedName>
-    <definedName name="curve_y1">'Reference'!$O$5:$O$34</definedName>
-    <definedName name="curve_x2">'Reference'!$H$5:$H$34</definedName>
-    <definedName name="curve_y2">'Reference'!$P$5:$P$34</definedName>
-    <definedName name="curve_x3">'Reference'!$I$5:$I$34</definedName>
-    <definedName name="curve_y3">'Reference'!$Q$5:$Q$34</definedName>
-    <definedName name="curve_x4">'Reference'!$J$5:$J$34</definedName>
-    <definedName name="curve_y4">'Reference'!$R$5:$R$34</definedName>
-    <definedName name="curve_x5">'Reference'!$K$5:$K$34</definedName>
-    <definedName name="curve_y5">'Reference'!$S$5:$S$34</definedName>
-    <definedName name="curve_x6">'Reference'!$L$5:$L$34</definedName>
-    <definedName name="curve_y6">'Reference'!$T$5:$T$34</definedName>
-    <definedName name="curve_x7">'Reference'!$M$5:$M$34</definedName>
-    <definedName name="curve_y7">'Reference'!$U$5:$U$34</definedName>
-    <definedName name="curve_x8">'Reference'!$N$5:$N$34</definedName>
-    <definedName name="curve_y8">'Reference'!$V$5:$V$34</definedName>
+    <definedName name="curve_key">'Reference'!$A$5:$A$33</definedName>
+    <definedName name="curve_x1">'Reference'!$G$5:$G$33</definedName>
+    <definedName name="curve_y1">'Reference'!$O$5:$O$33</definedName>
+    <definedName name="curve_x2">'Reference'!$H$5:$H$33</definedName>
+    <definedName name="curve_y2">'Reference'!$P$5:$P$33</definedName>
+    <definedName name="curve_x3">'Reference'!$I$5:$I$33</definedName>
+    <definedName name="curve_y3">'Reference'!$Q$5:$Q$33</definedName>
+    <definedName name="curve_x4">'Reference'!$J$5:$J$33</definedName>
+    <definedName name="curve_y4">'Reference'!$R$5:$R$33</definedName>
+    <definedName name="curve_x5">'Reference'!$K$5:$K$33</definedName>
+    <definedName name="curve_y5">'Reference'!$S$5:$S$33</definedName>
+    <definedName name="curve_x6">'Reference'!$L$5:$L$33</definedName>
+    <definedName name="curve_y6">'Reference'!$T$5:$T$33</definedName>
+    <definedName name="curve_x7">'Reference'!$M$5:$M$33</definedName>
+    <definedName name="curve_y7">'Reference'!$U$5:$U$33</definedName>
+    <definedName name="curve_x8">'Reference'!$N$5:$N$33</definedName>
+    <definedName name="curve_y8">'Reference'!$V$5:$V$33</definedName>
     <definedName name="idx_spring_pctimp2019ws">'Metrics'!$V$5</definedName>
     <definedName name="idx_spring_pctag2019ws">'Metrics'!$V$6</definedName>
     <definedName name="idx_spring_pctwet2019ws">'Metrics'!$V$7</definedName>
@@ -47,22 +47,21 @@
     <definedName name="idx_spring_phab_sinu">'Metrics'!$V$16</definedName>
     <definedName name="idx_spring_phab_xbka">'Metrics'!$V$17</definedName>
     <definedName name="idx_spring_phab_lrbs_use">'Metrics'!$V$18</definedName>
-    <definedName name="idx_spring_phab_lsub_dmm">'Metrics'!$V$19</definedName>
-    <definedName name="idx_spring_phab_lwdeqvolm100">'Metrics'!$V$20</definedName>
-    <definedName name="idx_spring_chem_chla">'Metrics'!$V$21</definedName>
-    <definedName name="idx_spring_phab_xcdenmid">'Metrics'!$V$22</definedName>
-    <definedName name="idx_spring_phab_xcmgw">'Metrics'!$V$23</definedName>
-    <definedName name="idx_spring_chem_ntl">'Metrics'!$V$24</definedName>
-    <definedName name="idx_spring_chem_ptl">'Metrics'!$V$25</definedName>
-    <definedName name="idx_spring_chem_cond">'Metrics'!$V$26</definedName>
-    <definedName name="idx_spring_chem_ph">'Metrics'!$V$27</definedName>
-    <definedName name="idx_spring_chem_turb">'Metrics'!$V$28</definedName>
-    <definedName name="idx_spring_phab_pct_fast">'Metrics'!$V$29</definedName>
-    <definedName name="idx_spring_phab_xfc_nat">'Metrics'!$V$30</definedName>
-    <definedName name="idx_spring_fish_nat_totlntax">'Metrics'!$V$31</definedName>
-    <definedName name="idx_spring_bent_ept_ntax">'Metrics'!$V$32</definedName>
-    <definedName name="idx_spring_bent_hprime">'Metrics'!$V$33</definedName>
-    <definedName name="idx_spring_nid_dams_1mi">'Metrics'!$V$34</definedName>
+    <definedName name="idx_spring_phab_lwdeqvolm100">'Metrics'!$V$19</definedName>
+    <definedName name="idx_spring_phab_lsub_dmm">'Metrics'!$V$20</definedName>
+    <definedName name="idx_spring_phab_xcdenmid">'Metrics'!$V$21</definedName>
+    <definedName name="idx_spring_phab_xcmgw">'Metrics'!$V$22</definedName>
+    <definedName name="idx_spring_chem_ntl">'Metrics'!$V$23</definedName>
+    <definedName name="idx_spring_chem_ptl">'Metrics'!$V$24</definedName>
+    <definedName name="idx_spring_chem_cond">'Metrics'!$V$25</definedName>
+    <definedName name="idx_spring_chem_ph">'Metrics'!$V$26</definedName>
+    <definedName name="idx_spring_chem_turb">'Metrics'!$V$27</definedName>
+    <definedName name="idx_spring_phab_pct_fast">'Metrics'!$V$28</definedName>
+    <definedName name="idx_spring_phab_xfc_nat">'Metrics'!$V$29</definedName>
+    <definedName name="idx_spring_fish_nat_totlntax">'Metrics'!$V$30</definedName>
+    <definedName name="idx_spring_bent_ept_ntax">'Metrics'!$V$31</definedName>
+    <definedName name="idx_spring_bent_hprime">'Metrics'!$V$32</definedName>
+    <definedName name="idx_spring_nid_dams_1mi">'Metrics'!$V$33</definedName>
     <definedName name="fs_catchment_hydrology">'Results'!$B$4</definedName>
     <definedName name="fs_surface_water_storage">'Results'!$B$5</definedName>
     <definedName name="fs_reach_inflow">'Results'!$B$6</definedName>
@@ -106,22 +105,21 @@
     <definedName name="in_spring_phab_sinu">'DEEP Score'!$E$28</definedName>
     <definedName name="in_spring_phab_xbka">'DEEP Score'!$E$29</definedName>
     <definedName name="in_spring_phab_lrbs_use">'DEEP Score'!$E$30</definedName>
-    <definedName name="in_spring_phab_lsub_dmm">'DEEP Score'!$E$32</definedName>
-    <definedName name="in_spring_phab_lwdeqvolm100">'DEEP Score'!$E$33</definedName>
-    <definedName name="in_spring_chem_chla">'DEEP Score'!$E$35</definedName>
-    <definedName name="in_spring_phab_xcdenmid">'DEEP Score'!$E$36</definedName>
-    <definedName name="in_spring_phab_xcmgw">'DEEP Score'!$E$37</definedName>
-    <definedName name="in_spring_chem_ntl">'DEEP Score'!$E$38</definedName>
-    <definedName name="in_spring_chem_ptl">'DEEP Score'!$E$39</definedName>
-    <definedName name="in_spring_chem_cond">'DEEP Score'!$E$40</definedName>
-    <definedName name="in_spring_chem_ph">'DEEP Score'!$E$41</definedName>
-    <definedName name="in_spring_chem_turb">'DEEP Score'!$E$42</definedName>
-    <definedName name="in_spring_phab_pct_fast">'DEEP Score'!$E$43</definedName>
-    <definedName name="in_spring_phab_xfc_nat">'DEEP Score'!$E$44</definedName>
-    <definedName name="in_spring_fish_nat_totlntax">'DEEP Score'!$E$45</definedName>
-    <definedName name="in_spring_bent_ept_ntax">'DEEP Score'!$E$46</definedName>
-    <definedName name="in_spring_bent_hprime">'DEEP Score'!$E$47</definedName>
-    <definedName name="in_spring_nid_dams_1mi">'DEEP Score'!$E$48</definedName>
+    <definedName name="in_spring_phab_lwdeqvolm100">'DEEP Score'!$E$32</definedName>
+    <definedName name="in_spring_phab_lsub_dmm">'DEEP Score'!$E$33</definedName>
+    <definedName name="in_spring_phab_xcdenmid">'DEEP Score'!$E$35</definedName>
+    <definedName name="in_spring_phab_xcmgw">'DEEP Score'!$E$36</definedName>
+    <definedName name="in_spring_chem_ntl">'DEEP Score'!$E$37</definedName>
+    <definedName name="in_spring_chem_ptl">'DEEP Score'!$E$38</definedName>
+    <definedName name="in_spring_chem_cond">'DEEP Score'!$E$39</definedName>
+    <definedName name="in_spring_chem_ph">'DEEP Score'!$E$40</definedName>
+    <definedName name="in_spring_chem_turb">'DEEP Score'!$E$41</definedName>
+    <definedName name="in_spring_phab_pct_fast">'DEEP Score'!$E$42</definedName>
+    <definedName name="in_spring_phab_xfc_nat">'DEEP Score'!$E$43</definedName>
+    <definedName name="in_spring_fish_nat_totlntax">'DEEP Score'!$E$44</definedName>
+    <definedName name="in_spring_bent_ept_ntax">'DEEP Score'!$E$45</definedName>
+    <definedName name="in_spring_bent_hprime">'DEEP Score'!$E$46</definedName>
+    <definedName name="in_spring_nid_dams_1mi">'DEEP Score'!$E$47</definedName>
     <definedName name="site_notes">'DEEP Score'!$A$64</definedName>
     <definedName name="meta_assessment_id">'Metadata'!$B$4</definedName>
     <definedName name="meta_assessment_name">'Metadata'!$B$5</definedName>
@@ -667,10 +665,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1531,10 +1529,10 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="45" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Reference condition. Reference condition is set by a fixed landscape-pressure screen, never by a score. 25 borrow comparable least-disturbed stations from a parent ecoregion, stating the level and the transfer risk. A metric that no basis supports is not scored, and the function it would have scored is reported as unassessed.</t>
+          <t>Reference condition. Reference condition is set by a fixed landscape-pressure screen, never by a score. 27 borrow comparable least-disturbed stations from a wider region, stating the region and the transfer risk. 22 of these curves carried forward unchanged from version 5. A metric that no basis supports is not scored, and the function it would have scored is reported as unassessed.</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1642,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Version 5 | USEPA NRSA 2013-24 (L3 ecoregion 71), StreamCurves regional analysis, methodology 0.13-provisional</t>
+          <t>Version 6 | USEPA NRSA 2013-24 (L3 ecoregion 71), StreamCurves regional analysis, methodology 0.14-provisional</t>
         </is>
       </c>
     </row>
@@ -2354,12 +2352,12 @@
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>Substrate size</t>
+          <t>Large wood volume</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>log mm</t>
+          <t>m3/100m</t>
         </is>
       </c>
       <c r="E32" s="14" t="n"/>
@@ -2382,12 +2380,12 @@
       <c r="B33" s="40" t="n"/>
       <c r="C33" s="41" t="inlineStr">
         <is>
-          <t>Large wood volume</t>
+          <t>Substrate size</t>
         </is>
       </c>
       <c r="D33" s="42" t="inlineStr">
         <is>
-          <t>m3/100m</t>
+          <t>log mm</t>
         </is>
       </c>
       <c r="E33" s="43" t="n"/>
@@ -2430,57 +2428,71 @@
           <t>Physicochemistry</t>
         </is>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B35" s="28" t="inlineStr">
         <is>
           <t>Light &amp; thermal regime</t>
         </is>
       </c>
-      <c r="C35" s="12" t="inlineStr">
-        <is>
-          <t>Chlorophyll a</t>
-        </is>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
-        <is>
-          <t>ug/L</t>
-        </is>
-      </c>
-      <c r="E35" s="14" t="n"/>
-      <c r="F35" s="15" t="inlineStr"/>
-      <c r="G35" s="16">
+      <c r="C35" s="29" t="inlineStr">
+        <is>
+          <t>Canopy density, mid-channel</t>
+        </is>
+      </c>
+      <c r="D35" s="30" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E35" s="31" t="n"/>
+      <c r="F35" s="32" t="inlineStr"/>
+      <c r="G35" s="33">
         <f>IF('Metrics'!$V$21="","",'Metrics'!$V$21)</f>
         <v/>
       </c>
-      <c r="H35" s="17">
+      <c r="H35" s="34">
         <f>IF('Results'!$B$16="","",'Results'!$B$16)</f>
         <v/>
       </c>
-      <c r="I35" s="18">
+      <c r="I35" s="35">
         <f>IF('DEEP Score'!$H$35="","",IF('DEEP Score'!$H$35&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$35&lt;=10,"Functioning At-Risk","Functioning")))</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="19" t="n"/>
-      <c r="B36" s="20" t="n"/>
-      <c r="C36" s="21" t="inlineStr">
-        <is>
-          <t>Canopy density, mid-channel</t>
-        </is>
-      </c>
-      <c r="D36" s="22" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E36" s="23" t="n"/>
-      <c r="F36" s="24" t="inlineStr"/>
-      <c r="G36" s="25">
+      <c r="A36" s="53" t="inlineStr">
+        <is>
+          <t>Physicochemistry</t>
+        </is>
+      </c>
+      <c r="B36" s="28" t="inlineStr">
+        <is>
+          <t>Carbon processing</t>
+        </is>
+      </c>
+      <c r="C36" s="29" t="inlineStr">
+        <is>
+          <t>Riparian veg cover, woody</t>
+        </is>
+      </c>
+      <c r="D36" s="30" t="inlineStr">
+        <is>
+          <t>frac</t>
+        </is>
+      </c>
+      <c r="E36" s="31" t="n"/>
+      <c r="F36" s="32" t="inlineStr"/>
+      <c r="G36" s="33">
         <f>IF('Metrics'!$V$22="","",'Metrics'!$V$22)</f>
         <v/>
       </c>
-      <c r="H36" s="20" t="n"/>
-      <c r="I36" s="26" t="n"/>
+      <c r="H36" s="34">
+        <f>IF('Results'!$B$17="","",'Results'!$B$17)</f>
+        <v/>
+      </c>
+      <c r="I36" s="35">
+        <f>IF('DEEP Score'!$H$36="","",IF('DEEP Score'!$H$36&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$36&lt;=10,"Functioning At-Risk","Functioning")))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="54" t="inlineStr">
@@ -2488,386 +2500,365 @@
           <t>Physicochemistry</t>
         </is>
       </c>
-      <c r="B37" s="28" t="inlineStr">
-        <is>
-          <t>Carbon processing</t>
-        </is>
-      </c>
-      <c r="C37" s="29" t="inlineStr">
-        <is>
-          <t>Riparian veg cover, woody</t>
-        </is>
-      </c>
-      <c r="D37" s="30" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Nutrient cycling</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>Total nitrogen</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>mg N/L</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="n"/>
+      <c r="F37" s="15" t="inlineStr"/>
+      <c r="G37" s="16">
+        <f>IF('Metrics'!$V$23="","",'Metrics'!$V$23)</f>
+        <v/>
+      </c>
+      <c r="H37" s="17">
+        <f>IF('Results'!$B$18="","",'Results'!$B$18)</f>
+        <v/>
+      </c>
+      <c r="I37" s="18">
+        <f>IF('DEEP Score'!$H$37="","",IF('DEEP Score'!$H$37&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$37&lt;=10,"Functioning At-Risk","Functioning")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="n"/>
+      <c r="B38" s="20" t="n"/>
+      <c r="C38" s="21" t="inlineStr">
+        <is>
+          <t>Total phosphorus</t>
+        </is>
+      </c>
+      <c r="D38" s="22" t="inlineStr">
+        <is>
+          <t>ug/L</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="n"/>
+      <c r="F38" s="24" t="inlineStr"/>
+      <c r="G38" s="25">
+        <f>IF('Metrics'!$V$24="","",'Metrics'!$V$24)</f>
+        <v/>
+      </c>
+      <c r="H38" s="20" t="n"/>
+      <c r="I38" s="26" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="54" t="inlineStr">
+        <is>
+          <t>Physicochemistry</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Water &amp; soil quality</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>Specific conductivity</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>uS/cm</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="n"/>
+      <c r="F39" s="15" t="inlineStr"/>
+      <c r="G39" s="16">
+        <f>IF('Metrics'!$V$25="","",'Metrics'!$V$25)</f>
+        <v/>
+      </c>
+      <c r="H39" s="17">
+        <f>IF('Results'!$B$19="","",'Results'!$B$19)</f>
+        <v/>
+      </c>
+      <c r="I39" s="18">
+        <f>IF('DEEP Score'!$H$39="","",IF('DEEP Score'!$H$39&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$39&lt;=10,"Functioning At-Risk","Functioning")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="39" t="n"/>
+      <c r="B40" s="40" t="n"/>
+      <c r="C40" s="41" t="inlineStr">
+        <is>
+          <t>pH</t>
+        </is>
+      </c>
+      <c r="D40" s="42" t="inlineStr">
+        <is>
+          <t>Std. Units</t>
+        </is>
+      </c>
+      <c r="E40" s="43" t="n"/>
+      <c r="F40" s="44" t="inlineStr"/>
+      <c r="G40" s="45">
+        <f>IF('Metrics'!$V$26="","",'Metrics'!$V$26)</f>
+        <v/>
+      </c>
+      <c r="H40" s="40" t="n"/>
+      <c r="I40" s="46" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="19" t="n"/>
+      <c r="B41" s="20" t="n"/>
+      <c r="C41" s="21" t="inlineStr">
+        <is>
+          <t>Turbidity</t>
+        </is>
+      </c>
+      <c r="D41" s="22" t="inlineStr">
+        <is>
+          <t>NTU</t>
+        </is>
+      </c>
+      <c r="E41" s="23" t="n"/>
+      <c r="F41" s="24" t="inlineStr"/>
+      <c r="G41" s="25">
+        <f>IF('Metrics'!$V$27="","",'Metrics'!$V$27)</f>
+        <v/>
+      </c>
+      <c r="H41" s="20" t="n"/>
+      <c r="I41" s="26" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="55" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>Habitat provision</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>Fast-water / riffle habitat</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="n"/>
+      <c r="F42" s="15" t="inlineStr"/>
+      <c r="G42" s="16">
+        <f>IF('Metrics'!$V$28="","",'Metrics'!$V$28)</f>
+        <v/>
+      </c>
+      <c r="H42" s="17">
+        <f>IF('Results'!$B$20="","",'Results'!$B$20)</f>
+        <v/>
+      </c>
+      <c r="I42" s="18">
+        <f>IF('DEEP Score'!$H$42="","",IF('DEEP Score'!$H$42&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$42&lt;=10,"Functioning At-Risk","Functioning")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="19" t="n"/>
+      <c r="B43" s="20" t="n"/>
+      <c r="C43" s="21" t="inlineStr">
+        <is>
+          <t>Natural fish cover</t>
+        </is>
+      </c>
+      <c r="D43" s="22" t="inlineStr">
         <is>
           <t>frac</t>
         </is>
       </c>
-      <c r="E37" s="31" t="n"/>
-      <c r="F37" s="32" t="inlineStr"/>
-      <c r="G37" s="33">
-        <f>IF('Metrics'!$V$23="","",'Metrics'!$V$23)</f>
-        <v/>
-      </c>
-      <c r="H37" s="34">
-        <f>IF('Results'!$B$17="","",'Results'!$B$17)</f>
-        <v/>
-      </c>
-      <c r="I37" s="35">
-        <f>IF('DEEP Score'!$H$37="","",IF('DEEP Score'!$H$37&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$37&lt;=10,"Functioning At-Risk","Functioning")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="53" t="inlineStr">
-        <is>
-          <t>Physicochemistry</t>
-        </is>
-      </c>
-      <c r="B38" s="11" t="inlineStr">
-        <is>
-          <t>Nutrient cycling</t>
-        </is>
-      </c>
-      <c r="C38" s="12" t="inlineStr">
-        <is>
-          <t>Total nitrogen</t>
-        </is>
-      </c>
-      <c r="D38" s="13" t="inlineStr">
-        <is>
-          <t>mg N/L</t>
-        </is>
-      </c>
-      <c r="E38" s="14" t="n"/>
-      <c r="F38" s="15" t="inlineStr"/>
-      <c r="G38" s="16">
-        <f>IF('Metrics'!$V$24="","",'Metrics'!$V$24)</f>
-        <v/>
-      </c>
-      <c r="H38" s="17">
-        <f>IF('Results'!$B$18="","",'Results'!$B$18)</f>
-        <v/>
-      </c>
-      <c r="I38" s="18">
-        <f>IF('DEEP Score'!$H$38="","",IF('DEEP Score'!$H$38&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$38&lt;=10,"Functioning At-Risk","Functioning")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="19" t="n"/>
-      <c r="B39" s="20" t="n"/>
-      <c r="C39" s="21" t="inlineStr">
-        <is>
-          <t>Total phosphorus</t>
-        </is>
-      </c>
-      <c r="D39" s="22" t="inlineStr">
-        <is>
-          <t>ug/L</t>
-        </is>
-      </c>
-      <c r="E39" s="23" t="n"/>
-      <c r="F39" s="24" t="inlineStr"/>
-      <c r="G39" s="25">
-        <f>IF('Metrics'!$V$25="","",'Metrics'!$V$25)</f>
-        <v/>
-      </c>
-      <c r="H39" s="20" t="n"/>
-      <c r="I39" s="26" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="53" t="inlineStr">
-        <is>
-          <t>Physicochemistry</t>
-        </is>
-      </c>
-      <c r="B40" s="11" t="inlineStr">
-        <is>
-          <t>Water &amp; soil quality</t>
-        </is>
-      </c>
-      <c r="C40" s="12" t="inlineStr">
-        <is>
-          <t>Specific conductivity</t>
-        </is>
-      </c>
-      <c r="D40" s="13" t="inlineStr">
-        <is>
-          <t>uS/cm</t>
-        </is>
-      </c>
-      <c r="E40" s="14" t="n"/>
-      <c r="F40" s="15" t="inlineStr"/>
-      <c r="G40" s="16">
-        <f>IF('Metrics'!$V$26="","",'Metrics'!$V$26)</f>
-        <v/>
-      </c>
-      <c r="H40" s="17">
-        <f>IF('Results'!$B$19="","",'Results'!$B$19)</f>
-        <v/>
-      </c>
-      <c r="I40" s="18">
-        <f>IF('DEEP Score'!$H$40="","",IF('DEEP Score'!$H$40&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$40&lt;=10,"Functioning At-Risk","Functioning")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="39" t="n"/>
-      <c r="B41" s="40" t="n"/>
-      <c r="C41" s="41" t="inlineStr">
-        <is>
-          <t>pH</t>
-        </is>
-      </c>
-      <c r="D41" s="42" t="inlineStr">
-        <is>
-          <t>Std. Units</t>
-        </is>
-      </c>
-      <c r="E41" s="43" t="n"/>
-      <c r="F41" s="44" t="inlineStr"/>
-      <c r="G41" s="45">
-        <f>IF('Metrics'!$V$27="","",'Metrics'!$V$27)</f>
-        <v/>
-      </c>
-      <c r="H41" s="40" t="n"/>
-      <c r="I41" s="46" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="19" t="n"/>
-      <c r="B42" s="20" t="n"/>
-      <c r="C42" s="21" t="inlineStr">
-        <is>
-          <t>Turbidity</t>
-        </is>
-      </c>
-      <c r="D42" s="22" t="inlineStr">
-        <is>
-          <t>NTU</t>
-        </is>
-      </c>
-      <c r="E42" s="23" t="n"/>
-      <c r="F42" s="24" t="inlineStr"/>
-      <c r="G42" s="25">
-        <f>IF('Metrics'!$V$28="","",'Metrics'!$V$28)</f>
-        <v/>
-      </c>
-      <c r="H42" s="20" t="n"/>
-      <c r="I42" s="26" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="55" t="inlineStr">
+      <c r="E43" s="23" t="n"/>
+      <c r="F43" s="24" t="inlineStr"/>
+      <c r="G43" s="25">
+        <f>IF('Metrics'!$V$29="","",'Metrics'!$V$29)</f>
+        <v/>
+      </c>
+      <c r="H43" s="20" t="n"/>
+      <c r="I43" s="26" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="56" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="B43" s="11" t="inlineStr">
-        <is>
-          <t>Habitat provision</t>
-        </is>
-      </c>
-      <c r="C43" s="12" t="inlineStr">
-        <is>
-          <t>Fast-water / riffle habitat</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E43" s="14" t="n"/>
-      <c r="F43" s="15" t="inlineStr"/>
-      <c r="G43" s="16">
-        <f>IF('Metrics'!$V$29="","",'Metrics'!$V$29)</f>
-        <v/>
-      </c>
-      <c r="H43" s="17">
-        <f>IF('Results'!$B$20="","",'Results'!$B$20)</f>
-        <v/>
-      </c>
-      <c r="I43" s="18">
-        <f>IF('DEEP Score'!$H$43="","",IF('DEEP Score'!$H$43&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$43&lt;=10,"Functioning At-Risk","Functioning")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="19" t="n"/>
-      <c r="B44" s="20" t="n"/>
-      <c r="C44" s="21" t="inlineStr">
-        <is>
-          <t>Natural fish cover</t>
-        </is>
-      </c>
-      <c r="D44" s="22" t="inlineStr">
-        <is>
-          <t>frac</t>
-        </is>
-      </c>
-      <c r="E44" s="23" t="n"/>
-      <c r="F44" s="24" t="inlineStr"/>
-      <c r="G44" s="25">
+      <c r="B44" s="28" t="inlineStr">
+        <is>
+          <t>Population support</t>
+        </is>
+      </c>
+      <c r="C44" s="29" t="inlineStr">
+        <is>
+          <t>Native fish taxa richness</t>
+        </is>
+      </c>
+      <c r="D44" s="30" t="inlineStr"/>
+      <c r="E44" s="31" t="n"/>
+      <c r="F44" s="32" t="inlineStr"/>
+      <c r="G44" s="33">
         <f>IF('Metrics'!$V$30="","",'Metrics'!$V$30)</f>
         <v/>
       </c>
-      <c r="H44" s="20" t="n"/>
-      <c r="I44" s="26" t="n"/>
+      <c r="H44" s="34">
+        <f>IF('Results'!$B$21="","",'Results'!$B$21)</f>
+        <v/>
+      </c>
+      <c r="I44" s="35">
+        <f>IF('DEEP Score'!$H$44="","",IF('DEEP Score'!$H$44&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$44&lt;=10,"Functioning At-Risk","Functioning")))</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="56" t="inlineStr">
+      <c r="A45" s="55" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="B45" s="28" t="inlineStr">
-        <is>
-          <t>Population support</t>
-        </is>
-      </c>
-      <c r="C45" s="29" t="inlineStr">
-        <is>
-          <t>Native fish taxa richness</t>
-        </is>
-      </c>
-      <c r="D45" s="30" t="inlineStr"/>
-      <c r="E45" s="31" t="n"/>
-      <c r="F45" s="32" t="inlineStr"/>
-      <c r="G45" s="33">
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>Community dynamics</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>EPT taxa richness</t>
+        </is>
+      </c>
+      <c r="D45" s="13" t="inlineStr"/>
+      <c r="E45" s="14" t="n"/>
+      <c r="F45" s="15" t="inlineStr"/>
+      <c r="G45" s="16">
         <f>IF('Metrics'!$V$31="","",'Metrics'!$V$31)</f>
         <v/>
       </c>
-      <c r="H45" s="34">
-        <f>IF('Results'!$B$21="","",'Results'!$B$21)</f>
-        <v/>
-      </c>
-      <c r="I45" s="35">
+      <c r="H45" s="17">
+        <f>IF('Results'!$B$22="","",'Results'!$B$22)</f>
+        <v/>
+      </c>
+      <c r="I45" s="18">
         <f>IF('DEEP Score'!$H$45="","",IF('DEEP Score'!$H$45&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$45&lt;=10,"Functioning At-Risk","Functioning")))</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="55" t="inlineStr">
+      <c r="A46" s="19" t="n"/>
+      <c r="B46" s="20" t="n"/>
+      <c r="C46" s="21" t="inlineStr">
+        <is>
+          <t>Shannon diversity (H')</t>
+        </is>
+      </c>
+      <c r="D46" s="22" t="inlineStr">
+        <is>
+          <t>H'</t>
+        </is>
+      </c>
+      <c r="E46" s="23" t="n"/>
+      <c r="F46" s="24" t="inlineStr"/>
+      <c r="G46" s="25">
+        <f>IF('Metrics'!$V$32="","",'Metrics'!$V$32)</f>
+        <v/>
+      </c>
+      <c r="H46" s="20" t="n"/>
+      <c r="I46" s="26" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="56" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="B46" s="11" t="inlineStr">
-        <is>
-          <t>Community dynamics</t>
-        </is>
-      </c>
-      <c r="C46" s="12" t="inlineStr">
-        <is>
-          <t>EPT taxa richness</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="inlineStr"/>
-      <c r="E46" s="14" t="n"/>
-      <c r="F46" s="15" t="inlineStr"/>
-      <c r="G46" s="16">
-        <f>IF('Metrics'!$V$32="","",'Metrics'!$V$32)</f>
-        <v/>
-      </c>
-      <c r="H46" s="17">
-        <f>IF('Results'!$B$22="","",'Results'!$B$22)</f>
-        <v/>
-      </c>
-      <c r="I46" s="18">
-        <f>IF('DEEP Score'!$H$46="","",IF('DEEP Score'!$H$46&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$46&lt;=10,"Functioning At-Risk","Functioning")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="19" t="n"/>
-      <c r="B47" s="20" t="n"/>
-      <c r="C47" s="21" t="inlineStr">
-        <is>
-          <t>Shannon diversity (H')</t>
-        </is>
-      </c>
-      <c r="D47" s="22" t="inlineStr">
-        <is>
-          <t>H'</t>
-        </is>
-      </c>
-      <c r="E47" s="23" t="n"/>
-      <c r="F47" s="24" t="inlineStr"/>
-      <c r="G47" s="25">
+      <c r="B47" s="28" t="inlineStr">
+        <is>
+          <t>Watershed connectivity</t>
+        </is>
+      </c>
+      <c r="C47" s="29" t="inlineStr">
+        <is>
+          <t>Mapped dams within one mile</t>
+        </is>
+      </c>
+      <c r="D47" s="30" t="inlineStr">
+        <is>
+          <t>dams</t>
+        </is>
+      </c>
+      <c r="E47" s="31" t="n"/>
+      <c r="F47" s="32" t="inlineStr"/>
+      <c r="G47" s="33">
         <f>IF('Metrics'!$V$33="","",'Metrics'!$V$33)</f>
         <v/>
       </c>
-      <c r="H47" s="20" t="n"/>
-      <c r="I47" s="26" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="56" t="inlineStr">
-        <is>
-          <t>Biology</t>
-        </is>
-      </c>
-      <c r="B48" s="28" t="inlineStr">
-        <is>
-          <t>Watershed connectivity</t>
-        </is>
-      </c>
-      <c r="C48" s="29" t="inlineStr">
-        <is>
-          <t>Mapped dams within one mile</t>
-        </is>
-      </c>
-      <c r="D48" s="30" t="inlineStr">
-        <is>
-          <t>dams</t>
-        </is>
-      </c>
-      <c r="E48" s="31" t="n"/>
-      <c r="F48" s="32" t="inlineStr"/>
-      <c r="G48" s="33">
-        <f>IF('Metrics'!$V$34="","",'Metrics'!$V$34)</f>
-        <v/>
-      </c>
-      <c r="H48" s="34">
+      <c r="H47" s="34">
         <f>IF('Results'!$B$23="","",'Results'!$B$23)</f>
         <v/>
       </c>
-      <c r="I48" s="35">
-        <f>IF('DEEP Score'!$H$48="","",IF('DEEP Score'!$H$48&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$48&lt;=10,"Functioning At-Risk","Functioning")))</f>
-        <v/>
+      <c r="I47" s="35">
+        <f>IF('DEEP Score'!$H$47="","",IF('DEEP Score'!$H$47&lt;=5,"Non-Functioning",IF('DEEP Score'!$H$47&lt;=10,"Functioning At-Risk","Functioning")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="57" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="57" t="inlineStr">
-        <is>
-          <t>Summary</t>
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>Sub-index (0 to 1)</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>Condition</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="inlineStr">
-        <is>
-          <t>Outcome</t>
-        </is>
-      </c>
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>Sub-index (0 to 1)</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="inlineStr">
-        <is>
-          <t>Condition</t>
-        </is>
+      <c r="A51" s="58" t="inlineStr">
+        <is>
+          <t>Physical</t>
+        </is>
+      </c>
+      <c r="B51" s="59">
+        <f>'Results'!$B$26</f>
+        <v/>
+      </c>
+      <c r="C51" s="42">
+        <f>IF('DEEP Score'!$B$51&lt;=0.39,"Non-Functioning",IF('DEEP Score'!$B$51&lt;=0.69,"Functioning At-Risk","Functioning"))</f>
+        <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="58" t="inlineStr">
         <is>
-          <t>Physical</t>
+          <t>Chemical</t>
         </is>
       </c>
       <c r="B52" s="59">
-        <f>'Results'!$B$26</f>
+        <f>'Results'!$B$27</f>
         <v/>
       </c>
       <c r="C52" s="42">
@@ -2878,11 +2869,11 @@
     <row r="53">
       <c r="A53" s="58" t="inlineStr">
         <is>
-          <t>Chemical</t>
+          <t>Biological</t>
         </is>
       </c>
       <c r="B53" s="59">
-        <f>'Results'!$B$27</f>
+        <f>'Results'!$B$28</f>
         <v/>
       </c>
       <c r="C53" s="42">
@@ -2890,14 +2881,14 @@
         <v/>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="58" t="inlineStr">
-        <is>
-          <t>Biological</t>
-        </is>
-      </c>
-      <c r="B54" s="59">
-        <f>'Results'!$B$28</f>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="60" t="inlineStr">
+        <is>
+          <t>Ecosystem Condition Index</t>
+        </is>
+      </c>
+      <c r="B54" s="61">
+        <f>'Results'!$B$29</f>
         <v/>
       </c>
       <c r="C54" s="42">
@@ -2905,67 +2896,64 @@
         <v/>
       </c>
     </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="60" t="inlineStr">
-        <is>
-          <t>Ecosystem Condition Index</t>
-        </is>
-      </c>
-      <c r="B55" s="61">
-        <f>'Results'!$B$29</f>
-        <v/>
-      </c>
-      <c r="C55" s="42">
-        <f>IF('DEEP Score'!$B$55&lt;=0.39,"Non-Functioning",IF('DEEP Score'!$B$55&lt;=0.69,"Functioning At-Risk","Functioning"))</f>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functions with a score: </t>
+        </is>
+      </c>
+      <c r="B55" s="4">
+        <f>COUNT('Results'!$B$4:$B$23)&amp;" of 20"</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Functions with a score: </t>
-        </is>
-      </c>
-      <c r="B56" s="4">
-        <f>COUNT('Results'!$B$4:$B$23)&amp;" of 20"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
           <t>This assessment covers 20 of 20 STAF functions.</t>
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="62" t="inlineStr">
+        <is>
+          <t>Withheld for insufficient reference support (not scored)</t>
+        </is>
+      </c>
+    </row>
     <row r="59">
-      <c r="A59" s="62" t="inlineStr">
-        <is>
-          <t>Withheld for insufficient reference support (not scored)</t>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Tolerant individuals (%) ~ HBI</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Community dynamics</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Tolerant individuals (%) ~ HBI</t>
+          <t>Benthic total taxa richness</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Community dynamics</t>
+          <t>Population support</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Benthic total taxa richness</t>
+          <t>Chlorophyll a</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Population support</t>
+          <t>Light and thermal regime</t>
         </is>
       </c>
     </row>
@@ -3044,71 +3032,67 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CB3B"/>
-  <mergeCells count="62">
+  <mergeCells count="58">
     <mergeCell ref="I18:I20"/>
     <mergeCell ref="H26:H27"/>
     <mergeCell ref="I30:I31"/>
+    <mergeCell ref="I45:I46"/>
     <mergeCell ref="A24:A25"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="H43:H44"/>
     <mergeCell ref="B12:B13"/>
-    <mergeCell ref="H38:H39"/>
-    <mergeCell ref="B40:B42"/>
+    <mergeCell ref="I39:I41"/>
     <mergeCell ref="B8:D8"/>
+    <mergeCell ref="A45:A46"/>
     <mergeCell ref="I16:I17"/>
-    <mergeCell ref="B46:B47"/>
     <mergeCell ref="A16:A17"/>
     <mergeCell ref="A32:A34"/>
     <mergeCell ref="H32:H34"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="B42:B43"/>
     <mergeCell ref="I26:I27"/>
     <mergeCell ref="I22:I23"/>
     <mergeCell ref="H18:H20"/>
     <mergeCell ref="I28:I29"/>
-    <mergeCell ref="H35:H36"/>
-    <mergeCell ref="I40:I42"/>
     <mergeCell ref="A12:A13"/>
     <mergeCell ref="A26:A27"/>
     <mergeCell ref="I12:I13"/>
-    <mergeCell ref="H46:H47"/>
     <mergeCell ref="H22:H23"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="H45:H46"/>
+    <mergeCell ref="I37:I38"/>
     <mergeCell ref="B28:B29"/>
     <mergeCell ref="B32:B34"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B24:B25"/>
     <mergeCell ref="I24:I25"/>
-    <mergeCell ref="A40:A42"/>
-    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="B37:B38"/>
     <mergeCell ref="A64:I69"/>
+    <mergeCell ref="A39:A41"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="H16:H17"/>
+    <mergeCell ref="A42:A43"/>
     <mergeCell ref="H12:H13"/>
-    <mergeCell ref="I38:I39"/>
+    <mergeCell ref="I42:I43"/>
     <mergeCell ref="H28:H29"/>
+    <mergeCell ref="H37:H38"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="H24:H25"/>
     <mergeCell ref="B18:B20"/>
     <mergeCell ref="B30:B31"/>
     <mergeCell ref="I32:I34"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="H40:H42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="B39:B41"/>
     <mergeCell ref="H30:H31"/>
+    <mergeCell ref="H39:H41"/>
     <mergeCell ref="B22:B23"/>
     <mergeCell ref="A28:A29"/>
+    <mergeCell ref="H42:H43"/>
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="B26:B27"/>
-    <mergeCell ref="I46:I47"/>
     <mergeCell ref="A18:A20"/>
     <mergeCell ref="A30:A31"/>
   </mergeCells>
-  <conditionalFormatting sqref="G12:G48">
+  <conditionalFormatting sqref="G12:G47">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(ISNUMBER(G12),G12&lt;=0.39)</formula>
     </cfRule>
@@ -3119,7 +3103,7 @@
       <formula>AND(ISNUMBER(G12),G12&gt;0.69)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H12:H48">
+  <conditionalFormatting sqref="H12:H47">
     <cfRule type="expression" priority="4" dxfId="0">
       <formula>AND(ISNUMBER(H12),H12&lt;=5)</formula>
     </cfRule>
@@ -3130,7 +3114,7 @@
       <formula>AND(ISNUMBER(H12),H12&gt;10)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I12:I48">
+  <conditionalFormatting sqref="I12:I47">
     <cfRule type="expression" priority="7" dxfId="0">
       <formula>I12="Non-Functioning"</formula>
     </cfRule>
@@ -3152,7 +3136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V34"/>
+  <dimension ref="A1:V33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -4563,7 +4547,7 @@
     <row r="19">
       <c r="A19" s="40" t="inlineStr">
         <is>
-          <t>Substrate size</t>
+          <t>Large wood volume</t>
         </is>
       </c>
       <c r="B19" s="73">
@@ -4575,11 +4559,11 @@
         <v/>
       </c>
       <c r="D19" s="73">
-        <f>"spring_phab_lsub_dmm|"&amp;'Metrics'!$C$19</f>
+        <f>"spring_phab_lwdeqvolm100|"&amp;'Metrics'!$C$19</f>
         <v/>
       </c>
       <c r="E19" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$19,curve_key,0),MATCH("spring_phab_lsub_dmm|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$19,curve_key,0),MATCH("spring_phab_lwdeqvolm100|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F19" s="73">
@@ -4654,7 +4638,7 @@
     <row r="20">
       <c r="A20" s="40" t="inlineStr">
         <is>
-          <t>Large wood volume</t>
+          <t>Substrate size</t>
         </is>
       </c>
       <c r="B20" s="73">
@@ -4666,11 +4650,11 @@
         <v/>
       </c>
       <c r="D20" s="73">
-        <f>"spring_phab_lwdeqvolm100|"&amp;'Metrics'!$C$20</f>
+        <f>"spring_phab_lsub_dmm|"&amp;'Metrics'!$C$20</f>
         <v/>
       </c>
       <c r="E20" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$20,curve_key,0),MATCH("spring_phab_lwdeqvolm100|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$20,curve_key,0),MATCH("spring_phab_lsub_dmm|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F20" s="73">
@@ -4745,7 +4729,7 @@
     <row r="21">
       <c r="A21" s="40" t="inlineStr">
         <is>
-          <t>Chlorophyll a</t>
+          <t>Canopy density, mid-channel</t>
         </is>
       </c>
       <c r="B21" s="73">
@@ -4757,11 +4741,11 @@
         <v/>
       </c>
       <c r="D21" s="73">
-        <f>"spring_chem_chla|"&amp;'Metrics'!$C$21</f>
+        <f>"spring_phab_xcdenmid|"&amp;'Metrics'!$C$21</f>
         <v/>
       </c>
       <c r="E21" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$21,curve_key,0),MATCH("spring_chem_chla|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$21,curve_key,0),MATCH("spring_phab_xcdenmid|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F21" s="73">
@@ -4836,7 +4820,7 @@
     <row r="22">
       <c r="A22" s="40" t="inlineStr">
         <is>
-          <t>Canopy density, mid-channel</t>
+          <t>Riparian veg cover, woody</t>
         </is>
       </c>
       <c r="B22" s="73">
@@ -4848,11 +4832,11 @@
         <v/>
       </c>
       <c r="D22" s="73">
-        <f>"spring_phab_xcdenmid|"&amp;'Metrics'!$C$22</f>
+        <f>"spring_phab_xcmgw|"&amp;'Metrics'!$C$22</f>
         <v/>
       </c>
       <c r="E22" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$22,curve_key,0),MATCH("spring_phab_xcdenmid|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$22,curve_key,0),MATCH("spring_phab_xcmgw|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F22" s="73">
@@ -4927,7 +4911,7 @@
     <row r="23">
       <c r="A23" s="40" t="inlineStr">
         <is>
-          <t>Riparian veg cover, woody</t>
+          <t>Total nitrogen</t>
         </is>
       </c>
       <c r="B23" s="73">
@@ -4939,11 +4923,11 @@
         <v/>
       </c>
       <c r="D23" s="73">
-        <f>"spring_phab_xcmgw|"&amp;'Metrics'!$C$23</f>
+        <f>"spring_chem_ntl|"&amp;'Metrics'!$C$23</f>
         <v/>
       </c>
       <c r="E23" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$23,curve_key,0),MATCH("spring_phab_xcmgw|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$23,curve_key,0),MATCH("spring_chem_ntl|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F23" s="73">
@@ -5018,7 +5002,7 @@
     <row r="24">
       <c r="A24" s="40" t="inlineStr">
         <is>
-          <t>Total nitrogen</t>
+          <t>Total phosphorus</t>
         </is>
       </c>
       <c r="B24" s="73">
@@ -5030,11 +5014,11 @@
         <v/>
       </c>
       <c r="D24" s="73">
-        <f>"spring_chem_ntl|"&amp;'Metrics'!$C$24</f>
+        <f>"spring_chem_ptl|"&amp;'Metrics'!$C$24</f>
         <v/>
       </c>
       <c r="E24" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$24,curve_key,0),MATCH("spring_chem_ntl|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$24,curve_key,0),MATCH("spring_chem_ptl|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F24" s="73">
@@ -5109,7 +5093,7 @@
     <row r="25">
       <c r="A25" s="40" t="inlineStr">
         <is>
-          <t>Total phosphorus</t>
+          <t>Specific conductivity</t>
         </is>
       </c>
       <c r="B25" s="73">
@@ -5121,11 +5105,11 @@
         <v/>
       </c>
       <c r="D25" s="73">
-        <f>"spring_chem_ptl|"&amp;'Metrics'!$C$25</f>
+        <f>"spring_chem_cond|"&amp;'Metrics'!$C$25</f>
         <v/>
       </c>
       <c r="E25" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$25,curve_key,0),MATCH("spring_chem_ptl|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$25,curve_key,0),MATCH("spring_chem_cond|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F25" s="73">
@@ -5200,7 +5184,7 @@
     <row r="26">
       <c r="A26" s="40" t="inlineStr">
         <is>
-          <t>Specific conductivity</t>
+          <t>pH</t>
         </is>
       </c>
       <c r="B26" s="73">
@@ -5212,11 +5196,11 @@
         <v/>
       </c>
       <c r="D26" s="73">
-        <f>"spring_chem_cond|"&amp;'Metrics'!$C$26</f>
+        <f>"spring_chem_ph|"&amp;'Metrics'!$C$26</f>
         <v/>
       </c>
       <c r="E26" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$26,curve_key,0),MATCH("spring_chem_cond|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$26,curve_key,0),MATCH("spring_chem_ph|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F26" s="73">
@@ -5291,7 +5275,7 @@
     <row r="27">
       <c r="A27" s="40" t="inlineStr">
         <is>
-          <t>pH</t>
+          <t>Turbidity</t>
         </is>
       </c>
       <c r="B27" s="73">
@@ -5303,11 +5287,11 @@
         <v/>
       </c>
       <c r="D27" s="73">
-        <f>"spring_chem_ph|"&amp;'Metrics'!$C$27</f>
+        <f>"spring_chem_turb|"&amp;'Metrics'!$C$27</f>
         <v/>
       </c>
       <c r="E27" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$27,curve_key,0),MATCH("spring_chem_ph|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$27,curve_key,0),MATCH("spring_chem_turb|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F27" s="73">
@@ -5382,7 +5366,7 @@
     <row r="28">
       <c r="A28" s="40" t="inlineStr">
         <is>
-          <t>Turbidity</t>
+          <t>Fast-water / riffle habitat</t>
         </is>
       </c>
       <c r="B28" s="73">
@@ -5394,11 +5378,11 @@
         <v/>
       </c>
       <c r="D28" s="73">
-        <f>"spring_chem_turb|"&amp;'Metrics'!$C$28</f>
+        <f>"spring_phab_pct_fast|"&amp;'Metrics'!$C$28</f>
         <v/>
       </c>
       <c r="E28" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$28,curve_key,0),MATCH("spring_chem_turb|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$28,curve_key,0),MATCH("spring_phab_pct_fast|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F28" s="73">
@@ -5473,7 +5457,7 @@
     <row r="29">
       <c r="A29" s="40" t="inlineStr">
         <is>
-          <t>Fast-water / riffle habitat</t>
+          <t>Natural fish cover</t>
         </is>
       </c>
       <c r="B29" s="73">
@@ -5485,11 +5469,11 @@
         <v/>
       </c>
       <c r="D29" s="73">
-        <f>"spring_phab_pct_fast|"&amp;'Metrics'!$C$29</f>
+        <f>"spring_phab_xfc_nat|"&amp;'Metrics'!$C$29</f>
         <v/>
       </c>
       <c r="E29" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$29,curve_key,0),MATCH("spring_phab_pct_fast|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$29,curve_key,0),MATCH("spring_phab_xfc_nat|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F29" s="73">
@@ -5564,7 +5548,7 @@
     <row r="30">
       <c r="A30" s="40" t="inlineStr">
         <is>
-          <t>Natural fish cover</t>
+          <t>Native fish taxa richness</t>
         </is>
       </c>
       <c r="B30" s="73">
@@ -5576,11 +5560,11 @@
         <v/>
       </c>
       <c r="D30" s="73">
-        <f>"spring_phab_xfc_nat|"&amp;'Metrics'!$C$30</f>
+        <f>"spring_fish_nat_totlntax|"&amp;'Metrics'!$C$30</f>
         <v/>
       </c>
       <c r="E30" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$30,curve_key,0),MATCH("spring_phab_xfc_nat|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$30,curve_key,0),MATCH("spring_fish_nat_totlntax|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F30" s="73">
@@ -5655,7 +5639,7 @@
     <row r="31">
       <c r="A31" s="40" t="inlineStr">
         <is>
-          <t>Native fish taxa richness</t>
+          <t>EPT taxa richness</t>
         </is>
       </c>
       <c r="B31" s="73">
@@ -5667,11 +5651,11 @@
         <v/>
       </c>
       <c r="D31" s="73">
-        <f>"spring_fish_nat_totlntax|"&amp;'Metrics'!$C$31</f>
+        <f>"spring_bent_ept_ntax|"&amp;'Metrics'!$C$31</f>
         <v/>
       </c>
       <c r="E31" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$31,curve_key,0),MATCH("spring_fish_nat_totlntax|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$31,curve_key,0),MATCH("spring_bent_ept_ntax|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F31" s="73">
@@ -5746,7 +5730,7 @@
     <row r="32">
       <c r="A32" s="40" t="inlineStr">
         <is>
-          <t>EPT taxa richness</t>
+          <t>Shannon diversity (H')</t>
         </is>
       </c>
       <c r="B32" s="73">
@@ -5758,11 +5742,11 @@
         <v/>
       </c>
       <c r="D32" s="73">
-        <f>"spring_bent_ept_ntax|"&amp;'Metrics'!$C$32</f>
+        <f>"spring_bent_hprime|"&amp;'Metrics'!$C$32</f>
         <v/>
       </c>
       <c r="E32" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$32,curve_key,0),MATCH("spring_bent_ept_ntax|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$32,curve_key,0),MATCH("spring_bent_hprime|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F32" s="73">
@@ -5837,7 +5821,7 @@
     <row r="33">
       <c r="A33" s="40" t="inlineStr">
         <is>
-          <t>Shannon diversity (H')</t>
+          <t>Mapped dams within one mile</t>
         </is>
       </c>
       <c r="B33" s="73">
@@ -5849,11 +5833,11 @@
         <v/>
       </c>
       <c r="D33" s="73">
-        <f>"spring_bent_hprime|"&amp;'Metrics'!$C$33</f>
+        <f>"spring_nid_dams_1mi|"&amp;'Metrics'!$C$33</f>
         <v/>
       </c>
       <c r="E33" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$33,curve_key,0),MATCH("spring_bent_hprime|",curve_key,0))</f>
+        <f>IFERROR(MATCH('Metrics'!$D$33,curve_key,0),MATCH("spring_nid_dams_1mi|",curve_key,0))</f>
         <v/>
       </c>
       <c r="F33" s="73">
@@ -5922,97 +5906,6 @@
       </c>
       <c r="V33" s="74">
         <f>IF(ISNUMBER('Metrics'!$B$33),MAX(0,MIN(1,IF('Metrics'!$B$33&lt;='Metrics'!$F$33,'Metrics'!$N$33,IF('Metrics'!$B$33&gt;='Metrics'!$M$33,'Metrics'!$U$33,IF('Metrics'!$B$33&lt;='Metrics'!$G$33,IF('Metrics'!$G$33-'Metrics'!$F$33&lt;=0,'Metrics'!$O$33,'Metrics'!$N$33+('Metrics'!$B$33-'Metrics'!$F$33)/('Metrics'!$G$33-'Metrics'!$F$33)*('Metrics'!$O$33-'Metrics'!$N$33)),IF('Metrics'!$B$33&lt;='Metrics'!$H$33,IF('Metrics'!$H$33-'Metrics'!$G$33&lt;=0,'Metrics'!$P$33,'Metrics'!$O$33+('Metrics'!$B$33-'Metrics'!$G$33)/('Metrics'!$H$33-'Metrics'!$G$33)*('Metrics'!$P$33-'Metrics'!$O$33)),IF('Metrics'!$B$33&lt;='Metrics'!$I$33,IF('Metrics'!$I$33-'Metrics'!$H$33&lt;=0,'Metrics'!$Q$33,'Metrics'!$P$33+('Metrics'!$B$33-'Metrics'!$H$33)/('Metrics'!$I$33-'Metrics'!$H$33)*('Metrics'!$Q$33-'Metrics'!$P$33)),IF('Metrics'!$B$33&lt;='Metrics'!$J$33,IF('Metrics'!$J$33-'Metrics'!$I$33&lt;=0,'Metrics'!$R$33,'Metrics'!$Q$33+('Metrics'!$B$33-'Metrics'!$I$33)/('Metrics'!$J$33-'Metrics'!$I$33)*('Metrics'!$R$33-'Metrics'!$Q$33)),IF('Metrics'!$B$33&lt;='Metrics'!$K$33,IF('Metrics'!$K$33-'Metrics'!$J$33&lt;=0,'Metrics'!$S$33,'Metrics'!$R$33+('Metrics'!$B$33-'Metrics'!$J$33)/('Metrics'!$K$33-'Metrics'!$J$33)*('Metrics'!$S$33-'Metrics'!$R$33)),IF('Metrics'!$B$33&lt;='Metrics'!$L$33,IF('Metrics'!$L$33-'Metrics'!$K$33&lt;=0,'Metrics'!$T$33,'Metrics'!$S$33+('Metrics'!$B$33-'Metrics'!$K$33)/('Metrics'!$L$33-'Metrics'!$K$33)*('Metrics'!$T$33-'Metrics'!$S$33)),IF('Metrics'!$M$33-'Metrics'!$L$33&lt;=0,'Metrics'!$U$33,'Metrics'!$T$33+('Metrics'!$B$33-'Metrics'!$L$33)/('Metrics'!$M$33-'Metrics'!$L$33)*('Metrics'!$U$33-'Metrics'!$T$33)))))))))))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="40" t="inlineStr">
-        <is>
-          <t>Mapped dams within one mile</t>
-        </is>
-      </c>
-      <c r="B34" s="73">
-        <f>IF('DEEP Score'!$E$48="","",'DEEP Score'!$E$48)</f>
-        <v/>
-      </c>
-      <c r="C34" s="73">
-        <f>""</f>
-        <v/>
-      </c>
-      <c r="D34" s="73">
-        <f>"spring_nid_dams_1mi|"&amp;'Metrics'!$C$34</f>
-        <v/>
-      </c>
-      <c r="E34" s="73">
-        <f>IFERROR(MATCH('Metrics'!$D$34,curve_key,0),MATCH("spring_nid_dams_1mi|",curve_key,0))</f>
-        <v/>
-      </c>
-      <c r="F34" s="73">
-        <f>INDEX(curve_x1,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="G34" s="73">
-        <f>INDEX(curve_x2,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="H34" s="73">
-        <f>INDEX(curve_x3,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="I34" s="73">
-        <f>INDEX(curve_x4,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="J34" s="73">
-        <f>INDEX(curve_x5,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="K34" s="73">
-        <f>INDEX(curve_x6,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="L34" s="73">
-        <f>INDEX(curve_x7,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="M34" s="73">
-        <f>INDEX(curve_x8,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="N34" s="73">
-        <f>INDEX(curve_y1,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="O34" s="73">
-        <f>INDEX(curve_y2,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="P34" s="73">
-        <f>INDEX(curve_y3,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="Q34" s="73">
-        <f>INDEX(curve_y4,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="R34" s="73">
-        <f>INDEX(curve_y5,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="S34" s="73">
-        <f>INDEX(curve_y6,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="T34" s="73">
-        <f>INDEX(curve_y7,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="U34" s="73">
-        <f>INDEX(curve_y8,'Metrics'!$E$34)</f>
-        <v/>
-      </c>
-      <c r="V34" s="74">
-        <f>IF(ISNUMBER('Metrics'!$B$34),MAX(0,MIN(1,IF('Metrics'!$B$34&lt;='Metrics'!$F$34,'Metrics'!$N$34,IF('Metrics'!$B$34&gt;='Metrics'!$M$34,'Metrics'!$U$34,IF('Metrics'!$B$34&lt;='Metrics'!$G$34,IF('Metrics'!$G$34-'Metrics'!$F$34&lt;=0,'Metrics'!$O$34,'Metrics'!$N$34+('Metrics'!$B$34-'Metrics'!$F$34)/('Metrics'!$G$34-'Metrics'!$F$34)*('Metrics'!$O$34-'Metrics'!$N$34)),IF('Metrics'!$B$34&lt;='Metrics'!$H$34,IF('Metrics'!$H$34-'Metrics'!$G$34&lt;=0,'Metrics'!$P$34,'Metrics'!$O$34+('Metrics'!$B$34-'Metrics'!$G$34)/('Metrics'!$H$34-'Metrics'!$G$34)*('Metrics'!$P$34-'Metrics'!$O$34)),IF('Metrics'!$B$34&lt;='Metrics'!$I$34,IF('Metrics'!$I$34-'Metrics'!$H$34&lt;=0,'Metrics'!$Q$34,'Metrics'!$P$34+('Metrics'!$B$34-'Metrics'!$H$34)/('Metrics'!$I$34-'Metrics'!$H$34)*('Metrics'!$Q$34-'Metrics'!$P$34)),IF('Metrics'!$B$34&lt;='Metrics'!$J$34,IF('Metrics'!$J$34-'Metrics'!$I$34&lt;=0,'Metrics'!$R$34,'Metrics'!$Q$34+('Metrics'!$B$34-'Metrics'!$I$34)/('Metrics'!$J$34-'Metrics'!$I$34)*('Metrics'!$R$34-'Metrics'!$Q$34)),IF('Metrics'!$B$34&lt;='Metrics'!$K$34,IF('Metrics'!$K$34-'Metrics'!$J$34&lt;=0,'Metrics'!$S$34,'Metrics'!$R$34+('Metrics'!$B$34-'Metrics'!$J$34)/('Metrics'!$K$34-'Metrics'!$J$34)*('Metrics'!$S$34-'Metrics'!$R$34)),IF('Metrics'!$B$34&lt;='Metrics'!$L$34,IF('Metrics'!$L$34-'Metrics'!$K$34&lt;=0,'Metrics'!$T$34,'Metrics'!$S$34+('Metrics'!$B$34-'Metrics'!$K$34)/('Metrics'!$L$34-'Metrics'!$K$34)*('Metrics'!$T$34-'Metrics'!$S$34)),IF('Metrics'!$M$34-'Metrics'!$L$34&lt;=0,'Metrics'!$U$34,'Metrics'!$T$34+('Metrics'!$B$34-'Metrics'!$L$34)/('Metrics'!$M$34-'Metrics'!$L$34)*('Metrics'!$U$34-'Metrics'!$T$34)))))))))))),"")</f>
         <v/>
       </c>
     </row>
@@ -6633,7 +6526,7 @@
         </is>
       </c>
       <c r="B16" s="73">
-        <f>IF(COUNT('DEEP Score'!G35:G36)=0,"",SUM('DEEP Score'!G35:G36)/COUNT('DEEP Score'!G35:G36)*15)</f>
+        <f>IF(COUNT('DEEP Score'!G35:G35)=0,"",SUM('DEEP Score'!G35:G35)/COUNT('DEEP Score'!G35:G35)*15)</f>
         <v/>
       </c>
       <c r="C16" s="40" t="n">
@@ -6677,7 +6570,7 @@
         </is>
       </c>
       <c r="B17" s="73">
-        <f>IF(COUNT('DEEP Score'!G37:G37)=0,"",SUM('DEEP Score'!G37:G37)/COUNT('DEEP Score'!G37:G37)*15)</f>
+        <f>IF(COUNT('DEEP Score'!G36:G36)=0,"",SUM('DEEP Score'!G36:G36)/COUNT('DEEP Score'!G36:G36)*15)</f>
         <v/>
       </c>
       <c r="C17" s="40" t="n">
@@ -6721,7 +6614,7 @@
         </is>
       </c>
       <c r="B18" s="73">
-        <f>IF(COUNT('DEEP Score'!G38:G39)=0,"",SUM('DEEP Score'!G38:G39)/COUNT('DEEP Score'!G38:G39)*15)</f>
+        <f>IF(COUNT('DEEP Score'!G37:G38)=0,"",SUM('DEEP Score'!G37:G38)/COUNT('DEEP Score'!G37:G38)*15)</f>
         <v/>
       </c>
       <c r="C18" s="40" t="n">
@@ -6765,7 +6658,7 @@
         </is>
       </c>
       <c r="B19" s="73">
-        <f>IF(COUNT('DEEP Score'!G40:G42)=0,"",SUM('DEEP Score'!G40:G42)/COUNT('DEEP Score'!G40:G42)*15)</f>
+        <f>IF(COUNT('DEEP Score'!G39:G41)=0,"",SUM('DEEP Score'!G39:G41)/COUNT('DEEP Score'!G39:G41)*15)</f>
         <v/>
       </c>
       <c r="C19" s="40" t="n">
@@ -6809,7 +6702,7 @@
         </is>
       </c>
       <c r="B20" s="73">
-        <f>IF(COUNT('DEEP Score'!G43:G44)=0,"",SUM('DEEP Score'!G43:G44)/COUNT('DEEP Score'!G43:G44)*15)</f>
+        <f>IF(COUNT('DEEP Score'!G42:G43)=0,"",SUM('DEEP Score'!G42:G43)/COUNT('DEEP Score'!G42:G43)*15)</f>
         <v/>
       </c>
       <c r="C20" s="40" t="n">
@@ -6853,7 +6746,7 @@
         </is>
       </c>
       <c r="B21" s="73">
-        <f>IF(COUNT('DEEP Score'!G45:G45)=0,"",SUM('DEEP Score'!G45:G45)/COUNT('DEEP Score'!G45:G45)*15)</f>
+        <f>IF(COUNT('DEEP Score'!G44:G44)=0,"",SUM('DEEP Score'!G44:G44)/COUNT('DEEP Score'!G44:G44)*15)</f>
         <v/>
       </c>
       <c r="C21" s="40" t="n">
@@ -6897,7 +6790,7 @@
         </is>
       </c>
       <c r="B22" s="73">
-        <f>IF(COUNT('DEEP Score'!G46:G47)=0,"",SUM('DEEP Score'!G46:G47)/COUNT('DEEP Score'!G46:G47)*15)</f>
+        <f>IF(COUNT('DEEP Score'!G45:G46)=0,"",SUM('DEEP Score'!G45:G46)/COUNT('DEEP Score'!G45:G46)*15)</f>
         <v/>
       </c>
       <c r="C22" s="40" t="n">
@@ -6941,7 +6834,7 @@
         </is>
       </c>
       <c r="B23" s="73">
-        <f>IF(COUNT('DEEP Score'!G48:G48)=0,"",SUM('DEEP Score'!G48:G48)/COUNT('DEEP Score'!G48:G48)*15)</f>
+        <f>IF(COUNT('DEEP Score'!G47:G47)=0,"",SUM('DEEP Score'!G47:G47)/COUNT('DEEP Score'!G47:G47)*15)</f>
         <v/>
       </c>
       <c r="C23" s="40" t="n">
@@ -7046,7 +6939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V43"/>
+  <dimension ref="A1:V42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -7204,7 +7097,7 @@
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
-          <t>Scored against a published criterion rather than against stations from this ecoregion. The criterion carries its own definition of reference, which need not match this assessment's.</t>
+          <t>Fixed criteria, the same in every region</t>
         </is>
       </c>
       <c r="G5" s="40" t="n">
@@ -7278,7 +7171,7 @@
       </c>
       <c r="F6" s="40" t="inlineStr">
         <is>
-          <t>Scored against a published criterion rather than against stations from this ecoregion. The criterion carries its own definition of reference, which need not match this assessment's.</t>
+          <t>Fixed criteria, the same in every region</t>
         </is>
       </c>
       <c r="G6" s="40" t="n">
@@ -7352,7 +7245,7 @@
       </c>
       <c r="F7" s="40" t="inlineStr">
         <is>
-          <t>37 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high</t>
+          <t>37 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high, carried forward from version 5</t>
         </is>
       </c>
       <c r="G7" s="40" t="n">
@@ -7426,7 +7319,7 @@
       </c>
       <c r="F8" s="40" t="inlineStr">
         <is>
-          <t>Scored against a published criterion rather than against stations from this ecoregion. The criterion carries its own definition of reference, which need not match this assessment's.</t>
+          <t>Fixed criteria, the same in every region</t>
         </is>
       </c>
       <c r="G8" s="40" t="n">
@@ -7500,7 +7393,7 @@
       </c>
       <c r="F9" s="40" t="inlineStr">
         <is>
-          <t>37 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high</t>
+          <t>37 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high, carried forward from version 5</t>
         </is>
       </c>
       <c r="G9" s="40" t="n">
@@ -7574,7 +7467,7 @@
       </c>
       <c r="F10" s="40" t="inlineStr">
         <is>
-          <t>Scored against a published criterion rather than against stations from this ecoregion. The criterion carries its own definition of reference, which need not match this assessment's.</t>
+          <t>Fixed criteria, the same in every region</t>
         </is>
       </c>
       <c r="G10" s="40" t="n">
@@ -7648,7 +7541,7 @@
       </c>
       <c r="F11" s="40" t="inlineStr">
         <is>
-          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high</t>
+          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high, carried forward from version 5</t>
         </is>
       </c>
       <c r="G11" s="40" t="n">
@@ -7722,7 +7615,7 @@
       </c>
       <c r="F12" s="40" t="inlineStr">
         <is>
-          <t>18 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high</t>
+          <t>18 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high, carried forward from version 5</t>
         </is>
       </c>
       <c r="G12" s="40" t="n">
@@ -7796,7 +7689,7 @@
       </c>
       <c r="F13" s="40" t="inlineStr">
         <is>
-          <t>27 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high</t>
+          <t>27 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high, carried forward from version 5</t>
         </is>
       </c>
       <c r="G13" s="40" t="n">
@@ -7870,7 +7763,7 @@
       </c>
       <c r="F14" s="40" t="inlineStr">
         <is>
-          <t>27 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate</t>
+          <t>27 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate, carried forward from version 5</t>
         </is>
       </c>
       <c r="G14" s="40" t="n">
@@ -7944,7 +7837,7 @@
       </c>
       <c r="F15" s="40" t="inlineStr">
         <is>
-          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate</t>
+          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate, carried forward from version 5</t>
         </is>
       </c>
       <c r="G15" s="40" t="n">
@@ -8018,7 +7911,7 @@
       </c>
       <c r="F16" s="40" t="inlineStr">
         <is>
-          <t>25 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high</t>
+          <t>25 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high, carried forward from version 5</t>
         </is>
       </c>
       <c r="G16" s="40" t="n">
@@ -8092,7 +7985,7 @@
       </c>
       <c r="F17" s="40" t="inlineStr">
         <is>
-          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate</t>
+          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate, carried forward from version 5</t>
         </is>
       </c>
       <c r="G17" s="40" t="n">
@@ -8166,7 +8059,7 @@
       </c>
       <c r="F18" s="40" t="inlineStr">
         <is>
-          <t>27 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high</t>
+          <t>27 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high, carried forward from version 5</t>
         </is>
       </c>
       <c r="G18" s="40" t="n">
@@ -8221,17 +8114,17 @@
     <row r="19">
       <c r="A19" s="40" t="inlineStr">
         <is>
-          <t>spring_phab_lsub_dmm|</t>
+          <t>spring_phab_lwdeqvolm100|</t>
         </is>
       </c>
       <c r="B19" s="40" t="inlineStr">
         <is>
-          <t>spring-phab-lsub-dmm</t>
+          <t>spring-phab-lwdeqvolm100</t>
         </is>
       </c>
       <c r="C19" s="40" t="inlineStr">
         <is>
-          <t>Substrate size</t>
+          <t>Large wood volume</t>
         </is>
       </c>
       <c r="D19" s="40" t="inlineStr"/>
@@ -8240,32 +8133,32 @@
       </c>
       <c r="F19" s="40" t="inlineStr">
         <is>
-          <t>27 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate</t>
+          <t>91 least-disturbed stations borrowed from NARS-9 region SAP under the regional screen (agriculture at most 37.8 percent), transfer risk high</t>
         </is>
       </c>
       <c r="G19" s="40" t="n">
-        <v>-1.944121440251668</v>
+        <v>0</v>
       </c>
       <c r="H19" s="40" t="n">
-        <v>-0.7447376449902852</v>
+        <v>0.07799999841621943</v>
       </c>
       <c r="I19" s="40" t="n">
-        <v>0.8544407486915588</v>
+        <v>0.181999996304512</v>
       </c>
       <c r="J19" s="40" t="n">
-        <v>2.053824543952942</v>
+        <v>4.620893001556396</v>
       </c>
       <c r="K19" s="40" t="n">
-        <v>2.413639682531357</v>
+        <v>5.952560903131962</v>
       </c>
       <c r="L19" s="40" t="n">
-        <v>2.413639682531357</v>
+        <v>5.952560903131962</v>
       </c>
       <c r="M19" s="40" t="n">
-        <v>2.413639682531357</v>
+        <v>5.952560903131962</v>
       </c>
       <c r="N19" s="40" t="n">
-        <v>2.413639682531357</v>
+        <v>5.952560903131962</v>
       </c>
       <c r="O19" s="40" t="n">
         <v>0</v>
@@ -8295,17 +8188,17 @@
     <row r="20">
       <c r="A20" s="40" t="inlineStr">
         <is>
-          <t>spring_phab_lwdeqvolm100|</t>
+          <t>spring_phab_lsub_dmm|</t>
         </is>
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>spring-phab-lwdeqvolm100</t>
+          <t>spring-phab-lsub-dmm</t>
         </is>
       </c>
       <c r="C20" s="40" t="inlineStr">
         <is>
-          <t>Large wood volume</t>
+          <t>Substrate size</t>
         </is>
       </c>
       <c r="D20" s="40" t="inlineStr"/>
@@ -8314,32 +8207,32 @@
       </c>
       <c r="F20" s="40" t="inlineStr">
         <is>
-          <t>29 least-disturbed stations borrowed from Level II ecoregion 8.3 (Southeastern Usa Plains), transfer risk moderate</t>
+          <t>27 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate, carried forward from version 5</t>
         </is>
       </c>
       <c r="G20" s="40" t="n">
-        <v>0</v>
+        <v>-1.944121440251668</v>
       </c>
       <c r="H20" s="40" t="n">
-        <v>0.2271428448813302</v>
+        <v>-0.7447376449902852</v>
       </c>
       <c r="I20" s="40" t="n">
-        <v>0.5299999713897705</v>
+        <v>0.8544407486915588</v>
       </c>
       <c r="J20" s="40" t="n">
-        <v>2.549999952316284</v>
+        <v>2.053824543952942</v>
       </c>
       <c r="K20" s="40" t="n">
-        <v>3.155999946594238</v>
+        <v>2.413639682531357</v>
       </c>
       <c r="L20" s="40" t="n">
-        <v>3.155999946594238</v>
+        <v>2.413639682531357</v>
       </c>
       <c r="M20" s="40" t="n">
-        <v>3.155999946594238</v>
+        <v>2.413639682531357</v>
       </c>
       <c r="N20" s="40" t="n">
-        <v>3.155999946594238</v>
+        <v>2.413639682531357</v>
       </c>
       <c r="O20" s="40" t="n">
         <v>0</v>
@@ -8369,17 +8262,17 @@
     <row r="21">
       <c r="A21" s="40" t="inlineStr">
         <is>
-          <t>spring_chem_chla|</t>
+          <t>spring_phab_xcdenmid|</t>
         </is>
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>spring-chem-chla</t>
+          <t>spring-phab-xcdenmid</t>
         </is>
       </c>
       <c r="C21" s="40" t="inlineStr">
         <is>
-          <t>Chlorophyll a</t>
+          <t>Canopy density, mid-channel</t>
         </is>
       </c>
       <c r="D21" s="40" t="inlineStr"/>
@@ -8388,72 +8281,72 @@
       </c>
       <c r="F21" s="40" t="inlineStr">
         <is>
-          <t>24 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high</t>
+          <t>27 least-disturbed stations borrowed from Level II ecoregion 8.3 (Southeastern Usa Plains), transfer risk moderate, carried forward from version 5</t>
         </is>
       </c>
       <c r="G21" s="40" t="n">
-        <v>0.1061549827456474</v>
+        <v>0</v>
       </c>
       <c r="H21" s="40" t="n">
-        <v>0.559349998831749</v>
+        <v>35.17952728271484</v>
       </c>
       <c r="I21" s="40" t="n">
-        <v>2.070000052452087</v>
+        <v>82.08556365966797</v>
       </c>
       <c r="J21" s="40" t="n">
-        <v>4.084200123945871</v>
+        <v>97.99465179443359</v>
       </c>
       <c r="K21" s="40" t="n">
-        <v>5.59485017756621</v>
+        <v>100</v>
       </c>
       <c r="L21" s="40" t="n">
-        <v>5.59485017756621</v>
+        <v>100</v>
       </c>
       <c r="M21" s="40" t="n">
-        <v>5.59485017756621</v>
+        <v>100</v>
       </c>
       <c r="N21" s="40" t="n">
-        <v>5.59485017756621</v>
+        <v>100</v>
       </c>
       <c r="O21" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P21" s="40" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="Q21" s="40" t="n">
         <v>0.7</v>
       </c>
       <c r="R21" s="40" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="S21" s="40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T21" s="40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U21" s="40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V21" s="40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="40" t="inlineStr">
         <is>
-          <t>spring_phab_xcdenmid|</t>
+          <t>spring_phab_xcmgw|</t>
         </is>
       </c>
       <c r="B22" s="40" t="inlineStr">
         <is>
-          <t>spring-phab-xcdenmid</t>
+          <t>spring-phab-xcmgw</t>
         </is>
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
-          <t>Canopy density, mid-channel</t>
+          <t>Riparian veg cover, woody</t>
         </is>
       </c>
       <c r="D22" s="40" t="inlineStr"/>
@@ -8462,32 +8355,32 @@
       </c>
       <c r="F22" s="40" t="inlineStr">
         <is>
-          <t>27 least-disturbed stations borrowed from Level II ecoregion 8.3 (Southeastern Usa Plains), transfer risk moderate</t>
+          <t>29 least-disturbed stations borrowed from Level II ecoregion 8.3 (Southeastern Usa Plains), transfer risk moderate, carried forward from version 5</t>
         </is>
       </c>
       <c r="G22" s="40" t="n">
         <v>0</v>
       </c>
       <c r="H22" s="40" t="n">
-        <v>35.17952728271484</v>
+        <v>0.3384740352630615</v>
       </c>
       <c r="I22" s="40" t="n">
-        <v>82.08556365966797</v>
+        <v>0.7897727489471436</v>
       </c>
       <c r="J22" s="40" t="n">
-        <v>97.99465179443359</v>
+        <v>1.610227227210999</v>
       </c>
       <c r="K22" s="40" t="n">
-        <v>100</v>
+        <v>1.856363570690155</v>
       </c>
       <c r="L22" s="40" t="n">
-        <v>100</v>
+        <v>1.856363570690155</v>
       </c>
       <c r="M22" s="40" t="n">
-        <v>100</v>
+        <v>1.856363570690155</v>
       </c>
       <c r="N22" s="40" t="n">
-        <v>100</v>
+        <v>1.856363570690155</v>
       </c>
       <c r="O22" s="40" t="n">
         <v>0</v>
@@ -8517,17 +8410,17 @@
     <row r="23">
       <c r="A23" s="40" t="inlineStr">
         <is>
-          <t>spring_phab_xcmgw|</t>
+          <t>spring_chem_ntl|</t>
         </is>
       </c>
       <c r="B23" s="40" t="inlineStr">
         <is>
-          <t>spring-phab-xcmgw</t>
+          <t>spring-chem-ntl</t>
         </is>
       </c>
       <c r="C23" s="40" t="inlineStr">
         <is>
-          <t>Riparian veg cover, woody</t>
+          <t>Total nitrogen</t>
         </is>
       </c>
       <c r="D23" s="40" t="inlineStr"/>
@@ -8536,72 +8429,72 @@
       </c>
       <c r="F23" s="40" t="inlineStr">
         <is>
-          <t>29 least-disturbed stations borrowed from Level II ecoregion 8.3 (Southeastern Usa Plains), transfer risk moderate</t>
+          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate, carried forward from version 5</t>
         </is>
       </c>
       <c r="G23" s="40" t="n">
-        <v>0</v>
+        <v>0.1203249990940094</v>
       </c>
       <c r="H23" s="40" t="n">
-        <v>0.3384740352630615</v>
+        <v>0.1765000000596046</v>
       </c>
       <c r="I23" s="40" t="n">
-        <v>0.7897727489471436</v>
+        <v>0.3637500032782555</v>
       </c>
       <c r="J23" s="40" t="n">
-        <v>1.610227227210999</v>
+        <v>0.6134166742364565</v>
       </c>
       <c r="K23" s="40" t="n">
-        <v>1.856363570690155</v>
+        <v>0.8006666774551074</v>
       </c>
       <c r="L23" s="40" t="n">
-        <v>1.856363570690155</v>
+        <v>0.8006666774551074</v>
       </c>
       <c r="M23" s="40" t="n">
-        <v>1.856363570690155</v>
+        <v>0.8006666774551074</v>
       </c>
       <c r="N23" s="40" t="n">
-        <v>1.856363570690155</v>
+        <v>0.8006666774551074</v>
       </c>
       <c r="O23" s="40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P23" s="40" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="Q23" s="40" t="n">
         <v>0.7</v>
       </c>
       <c r="R23" s="40" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="S23" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T23" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U23" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V23" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="40" t="inlineStr">
         <is>
-          <t>spring_chem_ntl|</t>
+          <t>spring_chem_ptl|</t>
         </is>
       </c>
       <c r="B24" s="40" t="inlineStr">
         <is>
-          <t>spring-chem-ntl</t>
+          <t>spring-chem-ptl</t>
         </is>
       </c>
       <c r="C24" s="40" t="inlineStr">
         <is>
-          <t>Total nitrogen</t>
+          <t>Total phosphorus</t>
         </is>
       </c>
       <c r="D24" s="40" t="inlineStr"/>
@@ -8610,32 +8503,32 @@
       </c>
       <c r="F24" s="40" t="inlineStr">
         <is>
-          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate</t>
+          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate, carried forward from version 5</t>
         </is>
       </c>
       <c r="G24" s="40" t="n">
-        <v>0.1203249990940094</v>
+        <v>4.193524861335755</v>
       </c>
       <c r="H24" s="40" t="n">
-        <v>0.1765000000596046</v>
+        <v>10.33924984931946</v>
       </c>
       <c r="I24" s="40" t="n">
-        <v>0.3637500032782555</v>
+        <v>30.82499980926514</v>
       </c>
       <c r="J24" s="40" t="n">
-        <v>0.6134166742364565</v>
+        <v>58.1393330891927</v>
       </c>
       <c r="K24" s="40" t="n">
-        <v>0.8006666774551074</v>
+        <v>78.6250830491384</v>
       </c>
       <c r="L24" s="40" t="n">
-        <v>0.8006666774551074</v>
+        <v>78.6250830491384</v>
       </c>
       <c r="M24" s="40" t="n">
-        <v>0.8006666774551074</v>
+        <v>78.6250830491384</v>
       </c>
       <c r="N24" s="40" t="n">
-        <v>0.8006666774551074</v>
+        <v>78.6250830491384</v>
       </c>
       <c r="O24" s="40" t="n">
         <v>1</v>
@@ -8665,17 +8558,17 @@
     <row r="25">
       <c r="A25" s="40" t="inlineStr">
         <is>
-          <t>spring_chem_ptl|</t>
+          <t>spring_chem_cond|</t>
         </is>
       </c>
       <c r="B25" s="40" t="inlineStr">
         <is>
-          <t>spring-chem-ptl</t>
+          <t>spring-chem-cond</t>
         </is>
       </c>
       <c r="C25" s="40" t="inlineStr">
         <is>
-          <t>Total phosphorus</t>
+          <t>Specific conductivity</t>
         </is>
       </c>
       <c r="D25" s="40" t="inlineStr"/>
@@ -8684,32 +8577,32 @@
       </c>
       <c r="F25" s="40" t="inlineStr">
         <is>
-          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate</t>
+          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high, carried forward from version 5</t>
         </is>
       </c>
       <c r="G25" s="40" t="n">
-        <v>4.193524861335755</v>
+        <v>19.16500043869019</v>
       </c>
       <c r="H25" s="40" t="n">
-        <v>10.33924984931946</v>
+        <v>35.87500095367432</v>
       </c>
       <c r="I25" s="40" t="n">
-        <v>30.82499980926514</v>
+        <v>91.57500267028809</v>
       </c>
       <c r="J25" s="40" t="n">
-        <v>58.1393330891927</v>
+        <v>165.8416716257731</v>
       </c>
       <c r="K25" s="40" t="n">
-        <v>78.6250830491384</v>
+        <v>221.5416733423869</v>
       </c>
       <c r="L25" s="40" t="n">
-        <v>78.6250830491384</v>
+        <v>221.5416733423869</v>
       </c>
       <c r="M25" s="40" t="n">
-        <v>78.6250830491384</v>
+        <v>221.5416733423869</v>
       </c>
       <c r="N25" s="40" t="n">
-        <v>78.6250830491384</v>
+        <v>221.5416733423869</v>
       </c>
       <c r="O25" s="40" t="n">
         <v>1</v>
@@ -8739,72 +8632,72 @@
     <row r="26">
       <c r="A26" s="40" t="inlineStr">
         <is>
-          <t>spring_chem_cond|</t>
+          <t>spring_chem_ph|</t>
         </is>
       </c>
       <c r="B26" s="40" t="inlineStr">
         <is>
-          <t>spring-chem-cond</t>
+          <t>spring-chem-ph</t>
         </is>
       </c>
       <c r="C26" s="40" t="inlineStr">
         <is>
-          <t>Specific conductivity</t>
+          <t>pH</t>
         </is>
       </c>
       <c r="D26" s="40" t="inlineStr"/>
       <c r="E26" s="40" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F26" s="40" t="inlineStr">
         <is>
-          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high</t>
+          <t>25 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate, carried forward from version 5</t>
         </is>
       </c>
       <c r="G26" s="40" t="n">
-        <v>19.16500043869019</v>
+        <v>6.130000591278076</v>
       </c>
       <c r="H26" s="40" t="n">
-        <v>35.87500095367432</v>
+        <v>6.62000036239624</v>
       </c>
       <c r="I26" s="40" t="n">
-        <v>91.57500267028809</v>
+        <v>6.938500213623047</v>
       </c>
       <c r="J26" s="40" t="n">
-        <v>165.8416716257731</v>
+        <v>7.110000133514404</v>
       </c>
       <c r="K26" s="40" t="n">
-        <v>221.5416733423869</v>
+        <v>7.599999904632568</v>
       </c>
       <c r="L26" s="40" t="n">
-        <v>221.5416733423869</v>
+        <v>7.771499824523926</v>
       </c>
       <c r="M26" s="40" t="n">
-        <v>221.5416733423869</v>
+        <v>8.089999675750732</v>
       </c>
       <c r="N26" s="40" t="n">
-        <v>221.5416733423869</v>
+        <v>8.579999446868896</v>
       </c>
       <c r="O26" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P26" s="40" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="Q26" s="40" t="n">
         <v>0.7</v>
       </c>
       <c r="R26" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="S26" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="T26" s="40" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="U26" s="40" t="n">
         <v>0.3</v>
-      </c>
-      <c r="S26" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="T26" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="U26" s="40" t="n">
-        <v>0</v>
       </c>
       <c r="V26" s="40" t="n">
         <v>0</v>
@@ -8813,72 +8706,72 @@
     <row r="27">
       <c r="A27" s="40" t="inlineStr">
         <is>
-          <t>spring_chem_ph|</t>
+          <t>spring_chem_turb|</t>
         </is>
       </c>
       <c r="B27" s="40" t="inlineStr">
         <is>
-          <t>spring-chem-ph</t>
+          <t>spring-chem-turb</t>
         </is>
       </c>
       <c r="C27" s="40" t="inlineStr">
         <is>
-          <t>pH</t>
+          <t>Turbidity</t>
         </is>
       </c>
       <c r="D27" s="40" t="inlineStr"/>
       <c r="E27" s="40" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F27" s="40" t="inlineStr">
         <is>
-          <t>25 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate</t>
+          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate, carried forward from version 5</t>
         </is>
       </c>
       <c r="G27" s="40" t="n">
-        <v>6.130000591278076</v>
+        <v>0.5915000706911087</v>
       </c>
       <c r="H27" s="40" t="n">
-        <v>6.62000036239624</v>
+        <v>1.730000048875809</v>
       </c>
       <c r="I27" s="40" t="n">
-        <v>6.938500213623047</v>
+        <v>5.524999976158142</v>
       </c>
       <c r="J27" s="40" t="n">
-        <v>7.110000133514404</v>
+        <v>10.58499987920125</v>
       </c>
       <c r="K27" s="40" t="n">
-        <v>7.599999904632568</v>
+        <v>14.37999980648359</v>
       </c>
       <c r="L27" s="40" t="n">
-        <v>7.771499824523926</v>
+        <v>14.37999980648359</v>
       </c>
       <c r="M27" s="40" t="n">
-        <v>8.089999675750732</v>
+        <v>14.37999980648359</v>
       </c>
       <c r="N27" s="40" t="n">
-        <v>8.579999446868896</v>
+        <v>14.37999980648359</v>
       </c>
       <c r="O27" s="40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P27" s="40" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="Q27" s="40" t="n">
         <v>0.7</v>
       </c>
       <c r="R27" s="40" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="S27" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T27" s="40" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="U27" s="40" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="V27" s="40" t="n">
         <v>0</v>
@@ -8887,17 +8780,17 @@
     <row r="28">
       <c r="A28" s="40" t="inlineStr">
         <is>
-          <t>spring_chem_turb|</t>
+          <t>spring_phab_pct_fast|</t>
         </is>
       </c>
       <c r="B28" s="40" t="inlineStr">
         <is>
-          <t>spring-chem-turb</t>
+          <t>spring-phab-pct-fast</t>
         </is>
       </c>
       <c r="C28" s="40" t="inlineStr">
         <is>
-          <t>Turbidity</t>
+          <t>Fast-water / riffle habitat</t>
         </is>
       </c>
       <c r="D28" s="40" t="inlineStr"/>
@@ -8906,72 +8799,72 @@
       </c>
       <c r="F28" s="40" t="inlineStr">
         <is>
-          <t>26 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate</t>
+          <t>27 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate, carried forward from version 5</t>
         </is>
       </c>
       <c r="G28" s="40" t="n">
-        <v>0.5915000706911087</v>
+        <v>0</v>
       </c>
       <c r="H28" s="40" t="n">
-        <v>1.730000048875809</v>
+        <v>1.642857159887041</v>
       </c>
       <c r="I28" s="40" t="n">
-        <v>5.524999976158142</v>
+        <v>3.833333373069763</v>
       </c>
       <c r="J28" s="40" t="n">
-        <v>10.58499987920125</v>
+        <v>27.75757598876953</v>
       </c>
       <c r="K28" s="40" t="n">
-        <v>14.37999980648359</v>
+        <v>34.93484877347946</v>
       </c>
       <c r="L28" s="40" t="n">
-        <v>14.37999980648359</v>
+        <v>34.93484877347946</v>
       </c>
       <c r="M28" s="40" t="n">
-        <v>14.37999980648359</v>
+        <v>34.93484877347946</v>
       </c>
       <c r="N28" s="40" t="n">
-        <v>14.37999980648359</v>
+        <v>34.93484877347946</v>
       </c>
       <c r="O28" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P28" s="40" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="Q28" s="40" t="n">
         <v>0.7</v>
       </c>
       <c r="R28" s="40" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="S28" s="40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T28" s="40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U28" s="40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V28" s="40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="40" t="inlineStr">
         <is>
-          <t>spring_phab_pct_fast|</t>
+          <t>spring_phab_xfc_nat|</t>
         </is>
       </c>
       <c r="B29" s="40" t="inlineStr">
         <is>
-          <t>spring-phab-pct-fast</t>
+          <t>spring-phab-xfc-nat</t>
         </is>
       </c>
       <c r="C29" s="40" t="inlineStr">
         <is>
-          <t>Fast-water / riffle habitat</t>
+          <t>Natural fish cover</t>
         </is>
       </c>
       <c r="D29" s="40" t="inlineStr"/>
@@ -8980,32 +8873,32 @@
       </c>
       <c r="F29" s="40" t="inlineStr">
         <is>
-          <t>27 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate</t>
+          <t>29 least-disturbed stations borrowed from Level II ecoregion 8.3 (Southeastern Usa Plains), transfer risk moderate, carried forward from version 5</t>
         </is>
       </c>
       <c r="G29" s="40" t="n">
         <v>0</v>
       </c>
       <c r="H29" s="40" t="n">
-        <v>1.642857159887041</v>
+        <v>0.07792208024433681</v>
       </c>
       <c r="I29" s="40" t="n">
-        <v>3.833333373069763</v>
+        <v>0.1818181872367859</v>
       </c>
       <c r="J29" s="40" t="n">
-        <v>27.75757598876953</v>
+        <v>0.6727272868156433</v>
       </c>
       <c r="K29" s="40" t="n">
-        <v>34.93484877347946</v>
+        <v>0.8200000166893006</v>
       </c>
       <c r="L29" s="40" t="n">
-        <v>34.93484877347946</v>
+        <v>0.8200000166893006</v>
       </c>
       <c r="M29" s="40" t="n">
-        <v>34.93484877347946</v>
+        <v>0.8200000166893006</v>
       </c>
       <c r="N29" s="40" t="n">
-        <v>34.93484877347946</v>
+        <v>0.8200000166893006</v>
       </c>
       <c r="O29" s="40" t="n">
         <v>0</v>
@@ -9035,17 +8928,17 @@
     <row r="30">
       <c r="A30" s="40" t="inlineStr">
         <is>
-          <t>spring_phab_xfc_nat|</t>
+          <t>spring_fish_nat_totlntax|</t>
         </is>
       </c>
       <c r="B30" s="40" t="inlineStr">
         <is>
-          <t>spring-phab-xfc-nat</t>
+          <t>spring-fish-nat-totlntax</t>
         </is>
       </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
-          <t>Natural fish cover</t>
+          <t>Native fish taxa richness</t>
         </is>
       </c>
       <c r="D30" s="40" t="inlineStr"/>
@@ -9054,32 +8947,32 @@
       </c>
       <c r="F30" s="40" t="inlineStr">
         <is>
-          <t>29 least-disturbed stations borrowed from Level II ecoregion 8.3 (Southeastern Usa Plains), transfer risk moderate</t>
+          <t>25 least-disturbed stations borrowed from NARS-9 region SAP under the regional screen (agriculture at most 37.8 percent), transfer risk moderate</t>
         </is>
       </c>
       <c r="G30" s="40" t="n">
         <v>0</v>
       </c>
       <c r="H30" s="40" t="n">
-        <v>0.07792208024433681</v>
+        <v>3.857142857142857</v>
       </c>
       <c r="I30" s="40" t="n">
-        <v>0.1818181872367859</v>
+        <v>9</v>
       </c>
       <c r="J30" s="40" t="n">
-        <v>0.6727272868156433</v>
+        <v>24</v>
       </c>
       <c r="K30" s="40" t="n">
-        <v>0.8200000166893006</v>
+        <v>28.5</v>
       </c>
       <c r="L30" s="40" t="n">
-        <v>0.8200000166893006</v>
+        <v>28.5</v>
       </c>
       <c r="M30" s="40" t="n">
-        <v>0.8200000166893006</v>
+        <v>28.5</v>
       </c>
       <c r="N30" s="40" t="n">
-        <v>0.8200000166893006</v>
+        <v>28.5</v>
       </c>
       <c r="O30" s="40" t="n">
         <v>0</v>
@@ -9109,17 +9002,17 @@
     <row r="31">
       <c r="A31" s="40" t="inlineStr">
         <is>
-          <t>spring_fish_nat_totlntax|</t>
+          <t>spring_bent_ept_ntax|</t>
         </is>
       </c>
       <c r="B31" s="40" t="inlineStr">
         <is>
-          <t>spring-fish-nat-totlntax</t>
+          <t>spring-bent-ept-ntax</t>
         </is>
       </c>
       <c r="C31" s="40" t="inlineStr">
         <is>
-          <t>Native fish taxa richness</t>
+          <t>EPT taxa richness</t>
         </is>
       </c>
       <c r="D31" s="40" t="inlineStr"/>
@@ -9128,32 +9021,32 @@
       </c>
       <c r="F31" s="40" t="inlineStr">
         <is>
-          <t>16 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk moderate</t>
+          <t>17 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high, carried forward from version 5</t>
         </is>
       </c>
       <c r="G31" s="40" t="n">
         <v>0</v>
       </c>
       <c r="H31" s="40" t="n">
-        <v>2.464285714285714</v>
+        <v>3.857142857142857</v>
       </c>
       <c r="I31" s="40" t="n">
-        <v>5.75</v>
+        <v>9</v>
       </c>
       <c r="J31" s="40" t="n">
-        <v>14.25</v>
+        <v>18</v>
       </c>
       <c r="K31" s="40" t="n">
-        <v>16.8</v>
+        <v>20.7</v>
       </c>
       <c r="L31" s="40" t="n">
-        <v>16.8</v>
+        <v>20.7</v>
       </c>
       <c r="M31" s="40" t="n">
-        <v>16.8</v>
+        <v>20.7</v>
       </c>
       <c r="N31" s="40" t="n">
-        <v>16.8</v>
+        <v>20.7</v>
       </c>
       <c r="O31" s="40" t="n">
         <v>0</v>
@@ -9183,17 +9076,17 @@
     <row r="32">
       <c r="A32" s="40" t="inlineStr">
         <is>
-          <t>spring_bent_ept_ntax|</t>
+          <t>spring_bent_hprime|</t>
         </is>
       </c>
       <c r="B32" s="40" t="inlineStr">
         <is>
-          <t>spring-bent-ept-ntax</t>
+          <t>spring-bent-hprime</t>
         </is>
       </c>
       <c r="C32" s="40" t="inlineStr">
         <is>
-          <t>EPT taxa richness</t>
+          <t>Shannon diversity (H')</t>
         </is>
       </c>
       <c r="D32" s="40" t="inlineStr"/>
@@ -9202,32 +9095,32 @@
       </c>
       <c r="F32" s="40" t="inlineStr">
         <is>
-          <t>17 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high</t>
+          <t>17 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high, carried forward from version 5</t>
         </is>
       </c>
       <c r="G32" s="40" t="n">
         <v>0</v>
       </c>
       <c r="H32" s="40" t="n">
-        <v>3.857142857142857</v>
+        <v>1.071428571428571</v>
       </c>
       <c r="I32" s="40" t="n">
-        <v>9</v>
+        <v>2.5</v>
       </c>
       <c r="J32" s="40" t="n">
-        <v>18</v>
+        <v>3.180000066757202</v>
       </c>
       <c r="K32" s="40" t="n">
-        <v>20.7</v>
+        <v>3.384000086784363</v>
       </c>
       <c r="L32" s="40" t="n">
-        <v>20.7</v>
+        <v>3.384000086784363</v>
       </c>
       <c r="M32" s="40" t="n">
-        <v>20.7</v>
+        <v>3.384000086784363</v>
       </c>
       <c r="N32" s="40" t="n">
-        <v>20.7</v>
+        <v>3.384000086784363</v>
       </c>
       <c r="O32" s="40" t="n">
         <v>0</v>
@@ -9257,181 +9150,107 @@
     <row r="33">
       <c r="A33" s="40" t="inlineStr">
         <is>
-          <t>spring_bent_hprime|</t>
+          <t>spring_nid_dams_1mi|</t>
         </is>
       </c>
       <c r="B33" s="40" t="inlineStr">
         <is>
-          <t>spring-bent-hprime</t>
+          <t>spring-nid-dams-1mi</t>
         </is>
       </c>
       <c r="C33" s="40" t="inlineStr">
         <is>
-          <t>Shannon diversity (H')</t>
+          <t>Mapped dams within one mile</t>
         </is>
       </c>
       <c r="D33" s="40" t="inlineStr"/>
       <c r="E33" s="40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F33" s="40" t="inlineStr">
         <is>
-          <t>17 least-disturbed stations borrowed from Level I ecoregion 8 (Eastern Temperate Forests), transfer risk high</t>
+          <t>Fixed criteria, the same in every region</t>
         </is>
       </c>
       <c r="G33" s="40" t="n">
         <v>0</v>
       </c>
       <c r="H33" s="40" t="n">
-        <v>1.071428571428571</v>
+        <v>1</v>
       </c>
       <c r="I33" s="40" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="J33" s="40" t="n">
-        <v>3.180000066757202</v>
+        <v>3</v>
       </c>
       <c r="K33" s="40" t="n">
-        <v>3.384000086784363</v>
+        <v>3</v>
       </c>
       <c r="L33" s="40" t="n">
-        <v>3.384000086784363</v>
+        <v>3</v>
       </c>
       <c r="M33" s="40" t="n">
-        <v>3.384000086784363</v>
+        <v>3</v>
       </c>
       <c r="N33" s="40" t="n">
-        <v>3.384000086784363</v>
+        <v>3</v>
       </c>
       <c r="O33" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="P33" s="40" t="n">
+        <v>0.545</v>
+      </c>
+      <c r="Q33" s="40" t="n">
+        <v>0.195</v>
+      </c>
+      <c r="R33" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="P33" s="40" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Q33" s="40" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="R33" s="40" t="n">
-        <v>1</v>
-      </c>
       <c r="S33" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T33" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U33" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V33" s="40" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="40" t="inlineStr">
-        <is>
-          <t>spring_nid_dams_1mi|</t>
-        </is>
-      </c>
-      <c r="B34" s="40" t="inlineStr">
-        <is>
-          <t>spring-nid-dams-1mi</t>
-        </is>
-      </c>
-      <c r="C34" s="40" t="inlineStr">
-        <is>
-          <t>Mapped dams within one mile</t>
-        </is>
-      </c>
-      <c r="D34" s="40" t="inlineStr"/>
-      <c r="E34" s="40" t="n">
-        <v>4</v>
-      </c>
-      <c r="F34" s="40" t="inlineStr">
-        <is>
-          <t>Scored against a published criterion rather than against stations from this ecoregion. The criterion carries its own definition of reference, which need not match this assessment's.</t>
-        </is>
-      </c>
-      <c r="G34" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="I34" s="40" t="n">
-        <v>2</v>
-      </c>
-      <c r="J34" s="40" t="n">
-        <v>3</v>
-      </c>
-      <c r="K34" s="40" t="n">
-        <v>3</v>
-      </c>
-      <c r="L34" s="40" t="n">
-        <v>3</v>
-      </c>
-      <c r="M34" s="40" t="n">
-        <v>3</v>
-      </c>
-      <c r="N34" s="40" t="n">
-        <v>3</v>
-      </c>
-      <c r="O34" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="P34" s="40" t="n">
-        <v>0.545</v>
-      </c>
-      <c r="Q34" s="40" t="n">
-        <v>0.195</v>
-      </c>
-      <c r="R34" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="S34" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="T34" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="U34" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="V34" s="40" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="62" t="inlineStr">
+    </row>
+    <row r="36">
+      <c r="A36" s="62" t="inlineStr">
         <is>
           <t>Curve sets by metric</t>
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="62" t="inlineStr">
+        <is>
+          <t>Condition classes</t>
+        </is>
+      </c>
+    </row>
     <row r="40">
-      <c r="A40" s="62" t="inlineStr">
-        <is>
-          <t>Condition classes</t>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Metric index: at or below 0.39 Non-Functioning, at or below 0.69 Functioning At-Risk, above Functioning.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Metric index: at or below 0.39 Non-Functioning, at or below 0.69 Functioning At-Risk, above Functioning.</t>
+          <t>Function score (0 to 15): at or below 5 Non-Functioning, at or below 10 Functioning At-Risk, above Functioning.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
-        <is>
-          <t>Function score (0 to 15): at or below 5 Non-Functioning, at or below 10 Functioning At-Risk, above Functioning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
         <is>
           <t>Outcome weights: a direct contribution counts 1, an indirect one 0.1.</t>
         </is>
@@ -9506,7 +9325,7 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -9525,7 +9344,7 @@
       </c>
       <c r="B8" s="40" t="inlineStr">
         <is>
-          <t>sha256:d339376ab846e645ef6ae9c7c41e9ea0c58f19cca552e72c7e686bf680a19f19</t>
+          <t>sha256:c7f3ba4aab6330c47fa23613a0ca1969469bd4b99a8f5b268498601311da0f73</t>
         </is>
       </c>
     </row>
@@ -9549,7 +9368,7 @@
       </c>
       <c r="B10" s="40" t="inlineStr">
         <is>
-          <t>USEPA NRSA 2013-24 (L3 ecoregion 71), StreamCurves regional analysis, methodology 0.13-provisional</t>
+          <t>USEPA NRSA 2013-24 (L3 ecoregion 71), StreamCurves regional analysis, methodology 0.14-provisional</t>
         </is>
       </c>
     </row>
@@ -9606,7 +9425,7 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16">

</xml_diff>